<commit_message>
feat(openspec): archive 2026-03-01-fix-rpt-xml-parsing and update chklog parsing logic
Archived the fix-rpt-xml-parsing change, added parsing_logic.md, updated chklog.py, and cleaned up older log files.
</commit_message>
<xml_diff>
--- a/input_data/GP程式修改記錄.xlsx
+++ b/input_data/GP程式修改記錄.xlsx
@@ -10,10 +10,10 @@
     <sheet name="2026" sheetId="21" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026'!$A$2:$Z$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026'!$A$2:$Z$2</definedName>
     <definedName name="_xlnm.Criteria" localSheetId="0">'2026'!$2:$2</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="145621"/>
 </workbook>
 </file>
 
@@ -393,9 +393,6 @@
     <t>GPQ-20260006_Bug</t>
   </si>
   <si>
-    <t>scxmt176</t>
-  </si>
-  <si>
     <t>銷售預測調整副程式</t>
   </si>
   <si>
@@ -1037,6 +1034,10 @@
   </si>
   <si>
     <t>GPQ-20250025_Bug</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>scxmt176_sub</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1049,11 +1050,11 @@
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="178" formatCode="0_);[Red]\(0\)"/>
-    <numFmt numFmtId="180" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="181" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="182" formatCode="[$$-1009]#,##0.00_);[Red]\([$$-1009]#,##0.00\)"/>
-    <numFmt numFmtId="183" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="0_);[Red]\(0\)"/>
+    <numFmt numFmtId="177" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="178" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="179" formatCode="[$$-1009]#,##0.00_);[Red]\([$$-1009]#,##0.00\)"/>
+    <numFmt numFmtId="180" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="81">
     <font>
@@ -2282,424 +2283,424 @@
     </border>
   </borders>
   <cellStyleXfs count="790">
-    <xf numFmtId="182" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="16" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="17" fillId="13" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="18" fillId="23" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="33" fillId="24" borderId="3">
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="14" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="16" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="17" fillId="13" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="18" fillId="23" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="33" fillId="24" borderId="3">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="20" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="21" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="22" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="23" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="24" fillId="7" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="25" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="27" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="12" fillId="0" borderId="0" applyBorder="0">
+    <xf numFmtId="179" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="20" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="21" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="22" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="23" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="24" fillId="7" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="25" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="27" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="13" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="12" fillId="0" borderId="0" applyBorder="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="28" fillId="13" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="30" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="10" fillId="0" borderId="0">
+    <xf numFmtId="179" fontId="28" fillId="13" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="30" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="10" fillId="0" borderId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="11" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="11" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="42" fillId="0" borderId="0"/>
-    <xf numFmtId="178" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="10" fillId="0" borderId="0">
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="11" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="11" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="42" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="10" fillId="0" borderId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="57" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="10" fillId="0" borderId="0">
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="57" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="10" fillId="0" borderId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="182" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="57" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="9" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="36" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="36" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="10" fillId="0" borderId="0">
+    <xf numFmtId="179" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="57" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="36" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="36" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="10" fillId="0" borderId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="58" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="35" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="58" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="35" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="180" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="177" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="59" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="59" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="51" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="34" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="33" fillId="25" borderId="3">
+    <xf numFmtId="179" fontId="59" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="59" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="51" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="34" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="33" fillId="25" borderId="3">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="60" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="53" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="61" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="48" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="62" fillId="48" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="62" fillId="48" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="45" fillId="13" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="42" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="60" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="53" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="61" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="48" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="62" fillId="48" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="62" fillId="48" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="45" fillId="13" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="42" fillId="0" borderId="0"/>
     <xf numFmtId="42" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="181" fontId="9" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="9" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="9" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="181" fontId="9" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="183" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="178" fontId="9" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="9" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="9" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="178" fontId="9" fillId="0" borderId="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="180" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="42" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="63" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="50" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="49" borderId="19" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="179" fontId="63" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="50" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="49" borderId="19" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="182" fontId="64" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="179" fontId="64" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="182" fontId="65" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="47" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="50" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="51" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="52" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="53" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="54" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="55" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="66" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="67" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="38" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="68" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="39" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="69" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="40" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="69" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="40" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="37" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="3" fillId="0" borderId="11">
+    <xf numFmtId="179" fontId="65" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="47" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="50" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="51" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="52" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="53" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="54" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="55" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="66" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="67" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="38" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="68" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="39" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="69" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="40" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="69" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="40" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="37" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="3" fillId="0" borderId="11">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="54" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="70" fillId="56" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="49" fillId="7" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="71" fillId="48" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="52" fillId="13" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="72" fillId="57" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="46" fillId="23" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="73" fillId="58" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="44" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="74" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="41" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="54" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="70" fillId="56" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="49" fillId="7" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="71" fillId="48" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="52" fillId="13" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="72" fillId="57" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="46" fillId="23" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="73" fillId="58" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="44" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="74" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="41" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -2708,31 +2709,31 @@
     <xf numFmtId="44" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="36" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="36" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="36" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="36" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="76" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="77" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="78" fillId="13" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="36" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="79" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="179" fontId="36" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="36" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="36" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="36" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="76" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="77" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="78" fillId="13" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="36" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="79" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
@@ -3360,400 +3361,400 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="14" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="16" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="17" fillId="13" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="18" fillId="23" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="20" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="21" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="22" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="23" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="24" fillId="7" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="25" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="27" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="12" fillId="0" borderId="0" applyBorder="0">
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="14" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="14" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="16" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="17" fillId="13" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="18" fillId="23" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="20" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="21" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="22" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="23" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="24" fillId="7" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="25" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="27" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="13" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="12" fillId="0" borderId="0" applyBorder="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="28" fillId="13" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="30" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="10" fillId="0" borderId="0">
+    <xf numFmtId="179" fontId="28" fillId="13" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="30" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="10" fillId="0" borderId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="11" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="11" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="42" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="10" fillId="0" borderId="0">
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="11" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="11" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="42" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="10" fillId="0" borderId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="57" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="10" fillId="0" borderId="0">
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="57" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="10" fillId="0" borderId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="182" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="57" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="9" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="36" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="36" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="10" fillId="0" borderId="0">
+    <xf numFmtId="179" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="57" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="36" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="36" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="10" fillId="0" borderId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="58" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="35" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="55" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="59" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="59" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="51" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="60" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="53" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="61" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="48" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="62" fillId="48" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="62" fillId="48" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="45" fillId="13" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="63" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="50" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="55" fillId="49" borderId="19" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="42" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="58" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="35" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="55" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="59" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="59" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="51" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="60" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="53" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="61" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="48" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="62" fillId="48" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="62" fillId="48" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="45" fillId="13" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="63" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="50" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="55" fillId="49" borderId="19" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="42" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="182" fontId="64" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="179" fontId="64" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="182" fontId="65" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="47" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="50" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="51" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="52" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="53" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="54" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="56" fillId="55" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="43" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="66" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="67" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="38" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="68" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="39" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="69" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="40" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="69" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="40" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="37" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="3" fillId="0" borderId="11">
+    <xf numFmtId="179" fontId="65" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="47" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="50" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="51" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="52" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="53" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="54" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="56" fillId="55" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="43" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="66" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="67" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="38" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="68" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="39" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="69" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="40" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="69" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="40" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="37" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="3" fillId="0" borderId="11">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="54" fillId="0" borderId="0"/>
-    <xf numFmtId="182" fontId="70" fillId="56" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="49" fillId="7" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="71" fillId="48" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="52" fillId="13" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="72" fillId="57" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="46" fillId="23" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="73" fillId="58" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="44" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="182" fontId="74" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="41" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="54" fillId="0" borderId="0"/>
+    <xf numFmtId="179" fontId="70" fillId="56" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="49" fillId="7" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="71" fillId="48" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="52" fillId="13" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="72" fillId="57" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="46" fillId="23" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="73" fillId="58" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="44" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="179" fontId="74" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="41" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3790,58 +3791,58 @@
     </xf>
   </cellStyleXfs>
   <cellXfs count="34">
-    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="8" fillId="26" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="8" fillId="26" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="8" fillId="26" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="8" fillId="26" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="8" fillId="26" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="8" fillId="59" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="8" fillId="59" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="8" fillId="59" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="8" fillId="59" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="5" fillId="27" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="75" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="75" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="75" fillId="27" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="75" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="75" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="75" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="75" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="75" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3865,31 +3866,31 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="8" fillId="60" borderId="12" xfId="157" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="8" fillId="60" borderId="12" xfId="157" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="8" fillId="60" borderId="12" xfId="157" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="8" fillId="60" borderId="12" xfId="157" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="75" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="7" fillId="61" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="7" fillId="61" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="7" fillId="61" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="7" fillId="61" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="7" fillId="62" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="7" fillId="62" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="7" fillId="62" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="7" fillId="62" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="8" fillId="60" borderId="12" xfId="157" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="8" fillId="60" borderId="12" xfId="157" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="8" fillId="60" borderId="14" xfId="157" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="8" fillId="60" borderId="14" xfId="157" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5144,10 +5145,10 @@
         <v>54</v>
       </c>
       <c r="J2" s="26" t="s">
+        <v>107</v>
+      </c>
+      <c r="K2" s="25" t="s">
         <v>108</v>
-      </c>
-      <c r="K2" s="25" t="s">
-        <v>109</v>
       </c>
       <c r="L2" s="5" t="s">
         <v>5</v>
@@ -5290,10 +5291,10 @@
         <v>11</v>
       </c>
       <c r="F4" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="G4" s="10" t="s">
         <v>69</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>70</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>8</v>
@@ -5308,7 +5309,7 @@
         <v>8</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M4" s="9" t="s">
         <v>19</v>
@@ -5381,10 +5382,10 @@
         <v>1</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M5" s="9" t="s">
         <v>19</v>
@@ -5445,7 +5446,7 @@
         <v>37</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>8</v>
@@ -5457,10 +5458,10 @@
         <v>1</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="M6" s="9" t="s">
         <v>19</v>
@@ -5509,43 +5510,43 @@
         <v>46037</v>
       </c>
       <c r="C7" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="D7" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" s="9" t="s">
+      <c r="F7" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="G7" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="H7" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="I7" s="9" t="s">
         <v>79</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>80</v>
       </c>
       <c r="J7" s="9" t="s">
         <v>13</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="L7" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="M7" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="M7" s="9" t="s">
+      <c r="N7" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="N7" s="8" t="s">
-        <v>83</v>
-      </c>
       <c r="O7" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="P7" s="8">
         <v>46037</v>
@@ -5554,16 +5555,16 @@
         <v>46037</v>
       </c>
       <c r="R7" s="23" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="S7" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="T7" s="18">
         <v>0.2</v>
       </c>
       <c r="U7" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="V7" s="12"/>
       <c r="W7" s="9" t="s">
@@ -5585,43 +5586,43 @@
         <v>46037</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E8" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="F8" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="G8" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="H8" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="H8" s="9" t="s">
-        <v>88</v>
-      </c>
       <c r="I8" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J8" s="9" t="s">
         <v>13</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="L8" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="M8" s="9" t="s">
         <v>51</v>
       </c>
       <c r="N8" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="O8" s="9" t="s">
         <v>92</v>
-      </c>
-      <c r="O8" s="9" t="s">
-        <v>93</v>
       </c>
       <c r="P8" s="8">
         <v>46038</v>
@@ -5633,13 +5634,13 @@
         <v>20260114001</v>
       </c>
       <c r="S8" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="T8" s="18">
         <v>1</v>
       </c>
       <c r="U8" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="V8" s="12" t="s">
         <v>16</v>
@@ -5665,43 +5666,43 @@
         <v>46037</v>
       </c>
       <c r="C9" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="D9" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E9" s="9" t="s">
+      <c r="F9" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="G9" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="H9" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="I9" s="9" t="s">
         <v>98</v>
-      </c>
-      <c r="I9" s="9" t="s">
-        <v>99</v>
       </c>
       <c r="J9" s="9" t="s">
         <v>13</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L9" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M9" s="9" t="s">
         <v>51</v>
       </c>
       <c r="N9" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="O9" s="9" t="s">
         <v>101</v>
-      </c>
-      <c r="O9" s="9" t="s">
-        <v>102</v>
       </c>
       <c r="P9" s="8">
         <v>46038</v>
@@ -5713,13 +5714,13 @@
         <v>20260114001</v>
       </c>
       <c r="S9" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="T9" s="18">
         <v>4</v>
       </c>
       <c r="U9" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="V9" s="12" t="s">
         <v>56</v>
@@ -5745,43 +5746,43 @@
         <v>46037</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E10" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F10" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="G10" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="H10" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="I10" s="9" t="s">
         <v>98</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>99</v>
       </c>
       <c r="J10" s="9" t="s">
         <v>13</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M10" s="9" t="s">
         <v>51</v>
       </c>
       <c r="N10" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="O10" s="9" t="s">
         <v>105</v>
-      </c>
-      <c r="O10" s="9" t="s">
-        <v>106</v>
       </c>
       <c r="P10" s="8">
         <v>46038</v>
@@ -5790,16 +5791,16 @@
         <v>46037</v>
       </c>
       <c r="R10" s="23" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="S10" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="T10" s="18">
         <v>0.5</v>
       </c>
       <c r="U10" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="V10" s="12"/>
       <c r="W10" s="9" t="s">
@@ -5821,43 +5822,43 @@
         <v>46041</v>
       </c>
       <c r="C11" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="D11" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E11" s="9" t="s">
+      <c r="F11" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="G11" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="H11" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="I11" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="I11" s="9" t="s">
+      <c r="J11" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="K11" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="L11" s="10" t="s">
         <v>116</v>
-      </c>
-      <c r="J11" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="K11" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="L11" s="10" t="s">
-        <v>117</v>
       </c>
       <c r="M11" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N11" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="O11" s="9" t="s">
         <v>118</v>
-      </c>
-      <c r="O11" s="9" t="s">
-        <v>119</v>
       </c>
       <c r="P11" s="8">
         <v>46041</v>
@@ -5866,20 +5867,20 @@
         <v>46031</v>
       </c>
       <c r="R11" s="23" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="S11" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="T11" s="18">
         <v>1</v>
       </c>
       <c r="U11" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="V11" s="12"/>
       <c r="W11" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="X11" s="8">
         <v>46041</v>
@@ -5897,34 +5898,34 @@
         <v>46045</v>
       </c>
       <c r="C12" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="D12" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="9" t="s">
+      <c r="F12" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="G12" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="H12" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="I12" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="J12" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="I12" s="9" t="s">
+      <c r="K12" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="J12" s="9" t="s">
+      <c r="L12" s="10" t="s">
         <v>128</v>
-      </c>
-      <c r="K12" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="L12" s="10" t="s">
-        <v>129</v>
       </c>
       <c r="M12" s="9" t="s">
         <v>20</v>
@@ -5945,19 +5946,19 @@
         <v>40</v>
       </c>
       <c r="S12" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="T12" s="18">
         <v>3</v>
       </c>
       <c r="U12" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="V12" s="12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="W12" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="X12" s="8">
         <v>46045</v>
@@ -5977,40 +5978,40 @@
         <v>46045</v>
       </c>
       <c r="C13" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E13" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="D13" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E13" s="9" t="s">
+      <c r="F13" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="G13" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="H13" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="I13" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="I13" s="9" t="s">
+      <c r="J13" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="K13" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="L13" s="10" t="s">
         <v>136</v>
-      </c>
-      <c r="J13" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="K13" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="L13" s="10" t="s">
-        <v>137</v>
       </c>
       <c r="M13" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N13" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="O13" s="9" t="s">
         <v>20</v>
@@ -6022,20 +6023,20 @@
         <v>46048</v>
       </c>
       <c r="R13" s="23" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="S13" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="T13" s="18">
         <v>6</v>
       </c>
       <c r="U13" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="V13" s="12"/>
       <c r="W13" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X13" s="8">
         <v>46048</v>
@@ -6053,40 +6054,40 @@
         <v>46048</v>
       </c>
       <c r="C14" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="D14" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>132</v>
-      </c>
       <c r="F14" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="G14" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="G14" s="10" t="s">
+      <c r="H14" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="J14" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="K14" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="L14" s="10" t="s">
         <v>142</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="I14" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="J14" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="K14" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="L14" s="10" t="s">
-        <v>143</v>
       </c>
       <c r="M14" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N14" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="O14" s="9" t="s">
         <v>20</v>
@@ -6098,20 +6099,20 @@
         <v>46048</v>
       </c>
       <c r="R14" s="23" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="S14" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="T14" s="18">
         <v>2</v>
       </c>
       <c r="U14" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="V14" s="12"/>
       <c r="W14" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="X14" s="8">
         <v>46048</v>
@@ -6129,40 +6130,40 @@
         <v>46048</v>
       </c>
       <c r="C15" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="D15" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E15" s="9" t="s">
+      <c r="F15" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="G15" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="G15" s="10" t="s">
+      <c r="H15" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="I15" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="I15" s="9" t="s">
+      <c r="J15" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="K15" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="L15" s="10" t="s">
         <v>149</v>
-      </c>
-      <c r="J15" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="K15" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="L15" s="10" t="s">
-        <v>150</v>
       </c>
       <c r="M15" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N15" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="O15" s="9" t="s">
         <v>20</v>
@@ -6177,19 +6178,19 @@
         <v>20260126001</v>
       </c>
       <c r="S15" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="T15" s="18">
         <v>6</v>
       </c>
       <c r="U15" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="V15" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="W15" s="9" t="s">
         <v>152</v>
-      </c>
-      <c r="W15" s="9" t="s">
-        <v>153</v>
       </c>
       <c r="X15" s="8">
         <v>46049</v>
@@ -6209,40 +6210,40 @@
         <v>46048</v>
       </c>
       <c r="C16" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="D16" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>145</v>
-      </c>
       <c r="F16" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="G16" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="G16" s="10" t="s">
+      <c r="H16" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="I16" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="J16" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="K16" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="L16" s="10" t="s">
         <v>155</v>
-      </c>
-      <c r="H16" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="I16" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="J16" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="K16" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="L16" s="10" t="s">
-        <v>156</v>
       </c>
       <c r="M16" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N16" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="O16" s="9" t="s">
         <v>20</v>
@@ -6257,19 +6258,19 @@
         <v>20260126001</v>
       </c>
       <c r="S16" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="T16" s="18">
         <v>6</v>
       </c>
       <c r="U16" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="V16" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="W16" s="9" t="s">
         <v>152</v>
-      </c>
-      <c r="W16" s="9" t="s">
-        <v>153</v>
       </c>
       <c r="X16" s="8">
         <v>46049</v>
@@ -6289,7 +6290,7 @@
         <v>46048</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D17" s="9" t="s">
         <v>39</v>
@@ -6301,28 +6302,28 @@
         <v>43</v>
       </c>
       <c r="G17" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="H17" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="I17" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="J17" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="K17" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="L17" s="10" t="s">
         <v>159</v>
-      </c>
-      <c r="I17" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="J17" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="K17" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="L17" s="10" t="s">
-        <v>160</v>
       </c>
       <c r="M17" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N17" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="O17" s="9" t="s">
         <v>20</v>
@@ -6337,16 +6338,16 @@
         <v>20260115004</v>
       </c>
       <c r="S17" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T17" s="18">
         <v>31</v>
       </c>
       <c r="U17" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="V17" s="12" t="s">
         <v>162</v>
-      </c>
-      <c r="V17" s="12" t="s">
-        <v>163</v>
       </c>
       <c r="W17" s="9"/>
       <c r="X17" s="8"/>
@@ -6365,7 +6366,7 @@
         <v>46048</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D18" s="9" t="s">
         <v>41</v>
@@ -6380,25 +6381,25 @@
         <v>41</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L18" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="M18" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N18" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="O18" s="9" t="s">
         <v>20</v>
@@ -6413,16 +6414,16 @@
         <v>20260115004</v>
       </c>
       <c r="S18" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T18" s="18">
         <v>19</v>
       </c>
       <c r="U18" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="V18" s="12" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="W18" s="9"/>
       <c r="X18" s="8"/>
@@ -6441,31 +6442,31 @@
         <v>46049</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D19" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E19" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="F19" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="G19" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="G19" s="10" t="s">
-        <v>168</v>
-      </c>
       <c r="H19" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I19" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L19" s="10" t="s">
         <v>52</v>
@@ -6474,7 +6475,7 @@
         <v>20</v>
       </c>
       <c r="N19" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="O19" s="9" t="s">
         <v>20</v>
@@ -6489,19 +6490,19 @@
         <v>20260115004</v>
       </c>
       <c r="S19" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T19" s="18">
         <v>1</v>
       </c>
       <c r="U19" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="V19" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="W19" s="9" t="s">
         <v>169</v>
-      </c>
-      <c r="W19" s="9" t="s">
-        <v>170</v>
       </c>
       <c r="X19" s="8">
         <v>46049</v>
@@ -6519,31 +6520,31 @@
         <v>46049</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F20" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="G20" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="G20" s="10" t="s">
-        <v>172</v>
-      </c>
       <c r="H20" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L20" s="10" t="s">
         <v>52</v>
@@ -6552,7 +6553,7 @@
         <v>20</v>
       </c>
       <c r="N20" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="O20" s="9" t="s">
         <v>20</v>
@@ -6567,19 +6568,19 @@
         <v>20260115004</v>
       </c>
       <c r="S20" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T20" s="18">
         <v>1</v>
       </c>
       <c r="U20" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="V20" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="W20" s="9" t="s">
         <v>169</v>
-      </c>
-      <c r="W20" s="9" t="s">
-        <v>170</v>
       </c>
       <c r="X20" s="8">
         <v>46049</v>
@@ -6597,31 +6598,31 @@
         <v>46049</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F21" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="G21" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="G21" s="10" t="s">
-        <v>174</v>
-      </c>
       <c r="H21" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L21" s="10" t="s">
         <v>52</v>
@@ -6630,7 +6631,7 @@
         <v>20</v>
       </c>
       <c r="N21" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="O21" s="9" t="s">
         <v>20</v>
@@ -6645,19 +6646,19 @@
         <v>20260115004</v>
       </c>
       <c r="S21" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T21" s="18">
         <v>1</v>
       </c>
       <c r="U21" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="V21" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="W21" s="9" t="s">
         <v>169</v>
-      </c>
-      <c r="W21" s="9" t="s">
-        <v>170</v>
       </c>
       <c r="X21" s="8">
         <v>46049</v>
@@ -6675,31 +6676,31 @@
         <v>46049</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F22" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G22" s="10" t="s">
         <v>175</v>
       </c>
-      <c r="G22" s="10" t="s">
-        <v>176</v>
-      </c>
       <c r="H22" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="J22" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L22" s="10" t="s">
         <v>52</v>
@@ -6708,7 +6709,7 @@
         <v>20</v>
       </c>
       <c r="N22" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="O22" s="9" t="s">
         <v>20</v>
@@ -6723,19 +6724,19 @@
         <v>20260115004</v>
       </c>
       <c r="S22" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T22" s="18">
         <v>1</v>
       </c>
       <c r="U22" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="V22" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="W22" s="9" t="s">
         <v>169</v>
-      </c>
-      <c r="W22" s="9" t="s">
-        <v>170</v>
       </c>
       <c r="X22" s="8">
         <v>46049</v>
@@ -6753,31 +6754,31 @@
         <v>46049</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F23" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="G23" s="10" t="s">
         <v>177</v>
       </c>
-      <c r="G23" s="10" t="s">
-        <v>178</v>
-      </c>
       <c r="H23" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L23" s="10" t="s">
         <v>52</v>
@@ -6786,7 +6787,7 @@
         <v>20</v>
       </c>
       <c r="N23" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="O23" s="9" t="s">
         <v>20</v>
@@ -6801,19 +6802,19 @@
         <v>20260115004</v>
       </c>
       <c r="S23" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T23" s="18">
         <v>1</v>
       </c>
       <c r="U23" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="V23" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="W23" s="9" t="s">
         <v>169</v>
-      </c>
-      <c r="W23" s="9" t="s">
-        <v>170</v>
       </c>
       <c r="X23" s="8">
         <v>46049</v>
@@ -6831,34 +6832,34 @@
         <v>46052</v>
       </c>
       <c r="C24" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E24" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="D24" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E24" s="9" t="s">
+      <c r="F24" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="F24" s="9" t="s">
+      <c r="G24" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="G24" s="10" t="s">
+      <c r="H24" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="H24" s="9" t="s">
+      <c r="I24" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="I24" s="9" t="s">
+      <c r="J24" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="K24" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="L24" s="10" t="s">
         <v>184</v>
-      </c>
-      <c r="J24" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="K24" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="L24" s="10" t="s">
-        <v>185</v>
       </c>
       <c r="M24" s="9" t="s">
         <v>20</v>
@@ -6867,7 +6868,7 @@
         <v>15</v>
       </c>
       <c r="O24" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="P24" s="8">
         <v>46052</v>
@@ -6876,20 +6877,20 @@
         <v>46052</v>
       </c>
       <c r="R24" s="23" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="S24" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="T24" s="18">
         <v>2.5</v>
       </c>
       <c r="U24" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="V24" s="12"/>
       <c r="W24" s="9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="X24" s="8">
         <v>46052</v>
@@ -6907,43 +6908,43 @@
         <v>46056</v>
       </c>
       <c r="C25" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E25" s="9" t="s">
         <v>189</v>
       </c>
-      <c r="D25" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E25" s="9" t="s">
+      <c r="F25" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="F25" s="9" t="s">
+      <c r="G25" s="10" t="s">
         <v>191</v>
       </c>
-      <c r="G25" s="10" t="s">
+      <c r="H25" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="H25" s="9" t="s">
+      <c r="I25" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="I25" s="9" t="s">
+      <c r="J25" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="K25" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="L25" s="10" t="s">
         <v>194</v>
-      </c>
-      <c r="J25" s="9" t="s">
-        <v>194</v>
-      </c>
-      <c r="K25" s="9" t="s">
-        <v>194</v>
-      </c>
-      <c r="L25" s="10" t="s">
-        <v>195</v>
       </c>
       <c r="M25" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N25" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="O25" s="9" t="s">
         <v>196</v>
-      </c>
-      <c r="O25" s="9" t="s">
-        <v>197</v>
       </c>
       <c r="P25" s="8">
         <v>46059</v>
@@ -6952,22 +6953,22 @@
         <v>46058</v>
       </c>
       <c r="R25" s="23" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="S25" s="9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="T25" s="18">
         <v>6</v>
       </c>
       <c r="U25" s="9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="V25" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="W25" s="9" t="s">
         <v>199</v>
-      </c>
-      <c r="W25" s="9" t="s">
-        <v>200</v>
       </c>
       <c r="X25" s="8">
         <v>46058</v>
@@ -6987,31 +6988,31 @@
         <v>46059</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D26" s="13" t="s">
         <v>41</v>
       </c>
       <c r="E26" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="G26" s="15" t="s">
         <v>202</v>
       </c>
-      <c r="F26" s="13" t="s">
-        <v>202</v>
-      </c>
-      <c r="G26" s="15" t="s">
+      <c r="H26" s="13" t="s">
         <v>203</v>
       </c>
-      <c r="H26" s="13" t="s">
-        <v>204</v>
-      </c>
       <c r="I26" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="J26" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K26" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L26" s="15" t="s">
         <v>45</v>
@@ -7020,7 +7021,7 @@
         <v>20</v>
       </c>
       <c r="N26" s="16" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O26" s="13" t="s">
         <v>20</v>
@@ -7032,10 +7033,10 @@
         <v>46064</v>
       </c>
       <c r="R26" s="27" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="S26" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="T26" s="21">
         <v>3</v>
@@ -7044,7 +7045,7 @@
         <v>12</v>
       </c>
       <c r="V26" s="17" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="W26" s="13"/>
       <c r="X26" s="16"/>
@@ -7063,40 +7064,40 @@
         <v>46059</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D27" s="13" t="s">
         <v>36</v>
       </c>
       <c r="E27" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="F27" s="13" t="s">
         <v>208</v>
       </c>
-      <c r="F27" s="13" t="s">
+      <c r="G27" s="15" t="s">
         <v>209</v>
       </c>
-      <c r="G27" s="15" t="s">
+      <c r="H27" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="I27" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="J27" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="K27" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="L27" s="15" t="s">
         <v>210</v>
-      </c>
-      <c r="H27" s="13" t="s">
-        <v>206</v>
-      </c>
-      <c r="I27" s="13" t="s">
-        <v>206</v>
-      </c>
-      <c r="J27" s="13" t="s">
-        <v>204</v>
-      </c>
-      <c r="K27" s="13" t="s">
-        <v>204</v>
-      </c>
-      <c r="L27" s="15" t="s">
-        <v>211</v>
       </c>
       <c r="M27" s="13" t="s">
         <v>20</v>
       </c>
       <c r="N27" s="16" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O27" s="13" t="s">
         <v>20</v>
@@ -7108,10 +7109,10 @@
         <v>46064</v>
       </c>
       <c r="R27" s="27" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="S27" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="T27" s="21">
         <v>3</v>
@@ -7120,10 +7121,10 @@
         <v>12</v>
       </c>
       <c r="V27" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="W27" s="13" t="s">
         <v>212</v>
-      </c>
-      <c r="W27" s="13" t="s">
-        <v>213</v>
       </c>
       <c r="X27" s="16">
         <v>46064</v>
@@ -7143,40 +7144,40 @@
         <v>46059</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D28" s="13" t="s">
         <v>36</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F28" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="G28" s="15" t="s">
         <v>214</v>
       </c>
-      <c r="G28" s="15" t="s">
-        <v>215</v>
-      </c>
       <c r="H28" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="I28" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="J28" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K28" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L28" s="15" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="M28" s="13" t="s">
         <v>20</v>
       </c>
       <c r="N28" s="16" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O28" s="13" t="s">
         <v>20</v>
@@ -7188,10 +7189,10 @@
         <v>46064</v>
       </c>
       <c r="R28" s="27" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="S28" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="T28" s="21">
         <v>1</v>
@@ -7200,10 +7201,10 @@
         <v>12</v>
       </c>
       <c r="V28" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="W28" s="13" t="s">
         <v>212</v>
-      </c>
-      <c r="W28" s="13" t="s">
-        <v>213</v>
       </c>
       <c r="X28" s="16">
         <v>46064</v>
@@ -7223,40 +7224,40 @@
         <v>46059</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D29" s="13" t="s">
         <v>36</v>
       </c>
       <c r="E29" s="13" t="s">
+        <v>215</v>
+      </c>
+      <c r="F29" s="13" t="s">
         <v>216</v>
       </c>
-      <c r="F29" s="13" t="s">
+      <c r="G29" s="15" t="s">
         <v>217</v>
       </c>
-      <c r="G29" s="15" t="s">
-        <v>218</v>
-      </c>
       <c r="H29" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="I29" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="J29" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K29" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L29" s="15" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="M29" s="13" t="s">
         <v>20</v>
       </c>
       <c r="N29" s="16" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O29" s="13" t="s">
         <v>20</v>
@@ -7268,10 +7269,10 @@
         <v>46064</v>
       </c>
       <c r="R29" s="27" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="S29" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="T29" s="21">
         <v>1</v>
@@ -7280,10 +7281,10 @@
         <v>12</v>
       </c>
       <c r="V29" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="W29" s="13" t="s">
         <v>212</v>
-      </c>
-      <c r="W29" s="13" t="s">
-        <v>213</v>
       </c>
       <c r="X29" s="16">
         <v>46064</v>
@@ -7303,40 +7304,40 @@
         <v>46059</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D30" s="13" t="s">
         <v>36</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G30" s="15" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="I30" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="J30" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K30" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L30" s="15" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="M30" s="13" t="s">
         <v>20</v>
       </c>
       <c r="N30" s="16" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O30" s="13" t="s">
         <v>20</v>
@@ -7348,10 +7349,10 @@
         <v>46064</v>
       </c>
       <c r="R30" s="27" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="S30" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="T30" s="21">
         <v>1</v>
@@ -7360,10 +7361,10 @@
         <v>12</v>
       </c>
       <c r="V30" s="17" t="s">
+        <v>211</v>
+      </c>
+      <c r="W30" s="13" t="s">
         <v>212</v>
-      </c>
-      <c r="W30" s="13" t="s">
-        <v>213</v>
       </c>
       <c r="X30" s="16">
         <v>46064</v>
@@ -7383,40 +7384,40 @@
         <v>46065</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D31" s="13" t="s">
         <v>36</v>
       </c>
       <c r="E31" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="F31" s="13" t="s">
         <v>220</v>
       </c>
-      <c r="F31" s="13" t="s">
+      <c r="G31" s="15" t="s">
         <v>221</v>
       </c>
-      <c r="G31" s="15" t="s">
+      <c r="H31" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="H31" s="13" t="s">
+      <c r="I31" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="I31" s="13" t="s">
+      <c r="J31" s="13" t="s">
+        <v>222</v>
+      </c>
+      <c r="K31" s="13" t="s">
+        <v>222</v>
+      </c>
+      <c r="L31" s="15" t="s">
         <v>224</v>
-      </c>
-      <c r="J31" s="13" t="s">
-        <v>223</v>
-      </c>
-      <c r="K31" s="13" t="s">
-        <v>223</v>
-      </c>
-      <c r="L31" s="15" t="s">
-        <v>225</v>
       </c>
       <c r="M31" s="13" t="s">
         <v>20</v>
       </c>
       <c r="N31" s="16" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="O31" s="13" t="s">
         <v>20</v>
@@ -7428,22 +7429,22 @@
         <v>46065</v>
       </c>
       <c r="R31" s="27" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="S31" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="T31" s="21">
         <v>4</v>
       </c>
       <c r="U31" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="V31" s="17" t="s">
+        <v>227</v>
+      </c>
+      <c r="W31" s="13" t="s">
         <v>228</v>
-      </c>
-      <c r="W31" s="13" t="s">
-        <v>229</v>
       </c>
       <c r="X31" s="16">
         <v>46065</v>
@@ -10528,6 +10529,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:Z2"/>
   <mergeCells count="3">
     <mergeCell ref="A1:V1"/>
     <mergeCell ref="W1:Y1"/>

</xml_diff>

<commit_message>
V0.18-docs(README.md): update Directory Structure description
</commit_message>
<xml_diff>
--- a/input_data/GP程式修改記錄.xlsx
+++ b/input_data/GP程式修改記錄.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\2.AI_Study_by_google_antigravity\tiptop-prog-chg-chk\input_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{292963C9-DAE6-452D-9C89-2FF974A8CD09}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A82B0182-0DFD-47B1-97C8-2EADDD098D78}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="17325" windowHeight="9840" tabRatio="379" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="2026 (2)" sheetId="22" r:id="rId1"/>
+    <sheet name="2026" sheetId="21" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026 (2)'!$A$2:$Z$25</definedName>
-    <definedName name="_xlnm.Criteria" localSheetId="0">'2026 (2)'!$2:$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026'!$A$2:$Z$25</definedName>
+    <definedName name="_xlnm.Criteria" localSheetId="0">'2026'!$2:$2</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
@@ -29,7 +29,7 @@
     <author>annietsai</author>
   </authors>
   <commentList>
-    <comment ref="V2" authorId="0" shapeId="0" xr:uid="{085C19CF-652B-4D35-87F0-BB3B6B053A26}">
+    <comment ref="V2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
       <text>
         <r>
           <rPr>
@@ -144,7 +144,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="837" uniqueCount="272">
   <si>
     <t>Bug</t>
   </si>
@@ -379,11 +379,31 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>Y</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>新增「自動產生(MIS)」按鈕</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>MIS</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Annie</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>MGW-AFA-002-0 TIPTOP GP-資產異動操作手冊</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jacky</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -422,10 +442,34 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>將錯誤訊息增加說明存在已確認但未過帳的調撥單</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>Tony</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MIS</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Bug</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>CIM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>aimi109</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -434,6 +478,14 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>Y</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>GPQ-20250179_客製需求</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -454,6 +506,10 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>CIM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>cimi150</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -462,10 +518,26 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>跟RD虛擬料相關欄位控卡可否鎖上以防RD人員填寫時亂填</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>RD</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ava</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>GPQ-20260004_Bug</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -482,6 +554,10 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>Bug</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>改rpt</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -490,10 +566,18 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>GPQ-20260009_Bug</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>CIM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>saimt370</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -502,10 +586,34 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>Excel匯入時控卡不可輸入借貨倉(B,B_SMT)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>MIS</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Steven</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Bug</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jacky</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>MGW-AXC-002-0 TIPTOP GP-成本結算操作手冊</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -526,10 +634,22 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>Y</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>修正重工單要乘1.8</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>Jacky</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>GPQ-20260010_Bug</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -546,10 +666,30 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>修正產生xml時折讓單號問題</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>MIS</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Bug</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jacky</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>amdp250</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -566,6 +706,10 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>CXC</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>cxcr200</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -574,10 +718,30 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>顯示[工單型態(sfb02)]</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>MIS</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MGW-AXC-002-0 TIPTOP GP-成本結算操作手冊</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jacky</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>axcr200</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -598,7 +762,19 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>SA撰寫</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MIS</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -607,6 +783,10 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>SD撰寫</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>BI業績_OBM併入ODM業五_配套修改-SD(1.0)-20260107.xlsx</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -628,6 +808,10 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>Jacky</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>axmt800</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -664,6 +848,10 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>CFA</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>safat108</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -672,6 +860,14 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>資產在未生效盤點單中,但程式顯示的訊息不對</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -680,10 +876,22 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>Bug</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jacky</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>GPQ-20260003_功能改善</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>CBM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>cbmr670</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -692,7 +900,23 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>格式1[元件][主件][用量], 加上[主件機種][頂階否]</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MIS</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Steven</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -705,23 +929,51 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>Jacky</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>GPQ-20250169_功能改善</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>NA</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>SD</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MIS</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>cxmi200資料整理及訂單毛利率放行功能修改-SD(1.0)-20260203.xlsx</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>CXM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>cxmi200</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>部門型態類別毛利設定作業</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>依SD說明</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -730,6 +982,18 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>Jacky</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>axmt800</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>訂單變更</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>CSUB</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -754,14 +1018,34 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>控卡客戶別Bug修正</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>MIS</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Bug</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>MGW-ABM-002-0 TIPTOP GP-BOM作業操作手冊</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>Jacky</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>GPQ-20250025_Bug</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -770,6 +1054,10 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>CIM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>scimi150_sub</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -778,6 +1066,14 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>1.各廠區單身資料僅接受1筆 2.各廠區各產生一筆承認序號</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -786,10 +1082,18 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>Bug</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>MGW-AIM-022-0 TIPTOP GP-料件資料建立操作手冊</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>Jacky</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>GPQ-20250051_功能改善</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -806,9 +1110,21 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>檢查停止交易的條件要改成同"檢查phase out"方式</t>
   </si>
   <si>
+    <t>MIS</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>20260224001</t>
   </si>
   <si>
@@ -828,6 +1144,14 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>Annie</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TW</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>cpmi255_sub</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -840,6 +1164,10 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>CPM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>apmt910</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -848,6 +1176,14 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>N</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Y</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>執行作業(KEY數量800)的時候會一直跳出警示視窗: "已有對應工單，只可變更交期，無法變更其他欄位"無法執行送簽;需強迫關閉,放棄…等</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -860,26 +1196,15 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>Bug</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TW</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>scxmt176_sub</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>GPQ-20260031_Bug</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>saxmt700</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>折讓單資料維護</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>雜項應收的折讓，預設[原始發票號碼]並控卡[原始發票號碼]必填。</t>
-  </si>
-  <si>
-    <t>Janet</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -3632,7 +3957,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3708,11 +4033,14 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="179" fontId="8" fillId="60" borderId="12" xfId="157" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="8" fillId="60" borderId="12" xfId="157" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="75" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="8" fillId="60" borderId="12" xfId="157" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="179" fontId="7" fillId="61" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4858,7 +5186,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{689D9BEF-339A-4E6C-8FED-59B169AF7E30}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
@@ -4888,36 +5216,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28"/>
-      <c r="P1" s="28"/>
-      <c r="Q1" s="28"/>
-      <c r="R1" s="28"/>
-      <c r="S1" s="28"/>
-      <c r="T1" s="28"/>
-      <c r="U1" s="28"/>
-      <c r="V1" s="28"/>
-      <c r="W1" s="29" t="s">
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
+      <c r="S1" s="29"/>
+      <c r="T1" s="29"/>
+      <c r="U1" s="29"/>
+      <c r="V1" s="29"/>
+      <c r="W1" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="X1" s="30"/>
-      <c r="Y1" s="30"/>
-      <c r="Z1" s="31" t="s">
+      <c r="X1" s="31"/>
+      <c r="Y1" s="31"/>
+      <c r="Z1" s="32" t="s">
         <v>51</v>
       </c>
     </row>
@@ -4943,17 +5271,17 @@
       <c r="G2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="H2" s="26" t="s">
+      <c r="H2" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="I2" s="26" t="s">
+      <c r="I2" s="25" t="s">
         <v>56</v>
       </c>
       <c r="J2" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="K2" s="26" t="s">
-        <v>92</v>
+        <v>110</v>
+      </c>
+      <c r="K2" s="25" t="s">
+        <v>111</v>
       </c>
       <c r="L2" s="5" t="s">
         <v>5</v>
@@ -4997,7 +5325,7 @@
       <c r="Y2" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="Z2" s="32"/>
+      <c r="Z2" s="33"/>
     </row>
     <row r="3" spans="1:26" s="1" customFormat="1" ht="30">
       <c r="A3" s="8">
@@ -5022,28 +5350,28 @@
         <v>63</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="J3" s="9" t="s">
         <v>13</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="L3" s="10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M3" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>14</v>
+        <v>67</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="P3" s="8">
         <v>46024</v>
@@ -5055,19 +5383,19 @@
         <v>21</v>
       </c>
       <c r="S3" s="9" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="T3" s="18">
         <v>6</v>
       </c>
       <c r="U3" s="9" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="V3" s="12" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="W3" s="9" t="s">
-        <v>17</v>
+        <v>70</v>
       </c>
       <c r="X3" s="8">
         <v>46024</v>
@@ -5087,7 +5415,7 @@
         <v>46034</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>36</v>
@@ -5096,10 +5424,10 @@
         <v>11</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>185</v>
+        <v>271</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>8</v>
@@ -5114,7 +5442,7 @@
         <v>8</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="M4" s="9" t="s">
         <v>19</v>
@@ -5163,7 +5491,7 @@
         <v>46034</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>36</v>
@@ -5187,10 +5515,10 @@
         <v>1</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>13</v>
+        <v>112</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="M5" s="9" t="s">
         <v>19</v>
@@ -5239,7 +5567,7 @@
         <v>46034</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>36</v>
@@ -5251,7 +5579,7 @@
         <v>37</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>8</v>
@@ -5263,10 +5591,10 @@
         <v>1</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>13</v>
+        <v>112</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="M6" s="9" t="s">
         <v>19</v>
@@ -5315,43 +5643,43 @@
         <v>46037</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>13</v>
+        <v>81</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>12</v>
+        <v>82</v>
       </c>
       <c r="J7" s="9" t="s">
         <v>13</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>13</v>
+        <v>81</v>
       </c>
       <c r="L7" s="10" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="N7" s="8" t="s">
-        <v>14</v>
+        <v>85</v>
       </c>
       <c r="O7" s="9" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="P7" s="8">
         <v>46037</v>
@@ -5360,16 +5688,16 @@
         <v>46037</v>
       </c>
       <c r="R7" s="23" t="s">
-        <v>40</v>
+        <v>86</v>
       </c>
       <c r="S7" s="9" t="s">
-        <v>12</v>
+        <v>82</v>
       </c>
       <c r="T7" s="18">
         <v>0.2</v>
       </c>
       <c r="U7" s="9" t="s">
-        <v>13</v>
+        <v>81</v>
       </c>
       <c r="V7" s="12"/>
       <c r="W7" s="9" t="s">
@@ -5391,43 +5719,43 @@
         <v>46037</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="J8" s="9" t="s">
         <v>13</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>13</v>
+        <v>91</v>
       </c>
       <c r="L8" s="10" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="M8" s="9" t="s">
         <v>53</v>
       </c>
       <c r="N8" s="8" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="O8" s="9" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="P8" s="8">
         <v>46038</v>
@@ -5439,13 +5767,13 @@
         <v>20260114001</v>
       </c>
       <c r="S8" s="9" t="s">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="T8" s="18">
         <v>1</v>
       </c>
       <c r="U8" s="9" t="s">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="V8" s="12" t="s">
         <v>16</v>
@@ -5471,43 +5799,43 @@
         <v>46037</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="D9" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="J9" s="9" t="s">
         <v>13</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="L9" s="10" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="M9" s="9" t="s">
         <v>53</v>
       </c>
       <c r="N9" s="8" t="s">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="O9" s="9" t="s">
-        <v>82</v>
+        <v>104</v>
       </c>
       <c r="P9" s="8">
         <v>46038</v>
@@ -5519,13 +5847,13 @@
         <v>20260114001</v>
       </c>
       <c r="S9" s="9" t="s">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="T9" s="18">
         <v>4</v>
       </c>
       <c r="U9" s="9" t="s">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="V9" s="12" t="s">
         <v>59</v>
@@ -5551,43 +5879,43 @@
         <v>46037</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="J10" s="9" t="s">
         <v>13</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="M10" s="9" t="s">
         <v>53</v>
       </c>
       <c r="N10" s="8" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="O10" s="9" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="P10" s="8">
         <v>46038</v>
@@ -5596,16 +5924,16 @@
         <v>46037</v>
       </c>
       <c r="R10" s="23" t="s">
-        <v>40</v>
+        <v>109</v>
       </c>
       <c r="S10" s="9" t="s">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="T10" s="18">
         <v>0.5</v>
       </c>
       <c r="U10" s="9" t="s">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="V10" s="12"/>
       <c r="W10" s="9" t="s">
@@ -5627,43 +5955,43 @@
         <v>46041</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>93</v>
+        <v>113</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>73</v>
+        <v>114</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>94</v>
+        <v>115</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>13</v>
+        <v>117</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>12</v>
+        <v>118</v>
       </c>
       <c r="J11" s="9" t="s">
-        <v>13</v>
+        <v>117</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>13</v>
+        <v>117</v>
       </c>
       <c r="L11" s="10" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="M11" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N11" s="8" t="s">
-        <v>14</v>
+        <v>120</v>
       </c>
       <c r="O11" s="9" t="s">
-        <v>20</v>
+        <v>121</v>
       </c>
       <c r="P11" s="8">
         <v>46041</v>
@@ -5672,20 +6000,20 @@
         <v>46031</v>
       </c>
       <c r="R11" s="23" t="s">
-        <v>40</v>
+        <v>122</v>
       </c>
       <c r="S11" s="9" t="s">
-        <v>12</v>
+        <v>118</v>
       </c>
       <c r="T11" s="18">
         <v>1</v>
       </c>
       <c r="U11" s="9" t="s">
-        <v>13</v>
+        <v>117</v>
       </c>
       <c r="V11" s="12"/>
       <c r="W11" s="9" t="s">
-        <v>17</v>
+        <v>123</v>
       </c>
       <c r="X11" s="8">
         <v>46041</v>
@@ -5703,34 +6031,34 @@
         <v>46045</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>98</v>
+        <v>125</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>99</v>
+        <v>126</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>100</v>
+        <v>127</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>101</v>
+        <v>128</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>12</v>
+        <v>129</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>12</v>
+        <v>129</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>13</v>
+        <v>130</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>13</v>
+        <v>130</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>102</v>
+        <v>131</v>
       </c>
       <c r="M12" s="9" t="s">
         <v>20</v>
@@ -5751,19 +6079,19 @@
         <v>40</v>
       </c>
       <c r="S12" s="9" t="s">
-        <v>12</v>
+        <v>129</v>
       </c>
       <c r="T12" s="18">
         <v>3</v>
       </c>
       <c r="U12" s="9" t="s">
-        <v>12</v>
+        <v>129</v>
       </c>
       <c r="V12" s="12" t="s">
-        <v>97</v>
+        <v>124</v>
       </c>
       <c r="W12" s="9" t="s">
-        <v>17</v>
+        <v>132</v>
       </c>
       <c r="X12" s="8">
         <v>46045</v>
@@ -5783,40 +6111,40 @@
         <v>46045</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>103</v>
+        <v>133</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>104</v>
+        <v>134</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>105</v>
+        <v>135</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>106</v>
+        <v>136</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>13</v>
+        <v>137</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>12</v>
+        <v>138</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>13</v>
+        <v>137</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>13</v>
+        <v>137</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>107</v>
+        <v>139</v>
       </c>
       <c r="M13" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N13" s="8" t="s">
-        <v>14</v>
+        <v>140</v>
       </c>
       <c r="O13" s="9" t="s">
         <v>20</v>
@@ -5828,20 +6156,20 @@
         <v>46048</v>
       </c>
       <c r="R13" s="23" t="s">
-        <v>40</v>
+        <v>141</v>
       </c>
       <c r="S13" s="9" t="s">
-        <v>12</v>
+        <v>138</v>
       </c>
       <c r="T13" s="18">
         <v>6</v>
       </c>
       <c r="U13" s="9" t="s">
-        <v>13</v>
+        <v>137</v>
       </c>
       <c r="V13" s="12"/>
       <c r="W13" s="9" t="s">
-        <v>17</v>
+        <v>142</v>
       </c>
       <c r="X13" s="8">
         <v>46048</v>
@@ -5859,40 +6187,40 @@
         <v>46048</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>103</v>
+        <v>133</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>104</v>
+        <v>134</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>108</v>
+        <v>143</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>109</v>
+        <v>144</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>13</v>
+        <v>137</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>12</v>
+        <v>138</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>13</v>
+        <v>137</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>13</v>
+        <v>137</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>110</v>
+        <v>145</v>
       </c>
       <c r="M14" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N14" s="8" t="s">
-        <v>14</v>
+        <v>140</v>
       </c>
       <c r="O14" s="9" t="s">
         <v>20</v>
@@ -5904,20 +6232,20 @@
         <v>46048</v>
       </c>
       <c r="R14" s="23" t="s">
-        <v>40</v>
+        <v>141</v>
       </c>
       <c r="S14" s="9" t="s">
-        <v>12</v>
+        <v>138</v>
       </c>
       <c r="T14" s="18">
         <v>2</v>
       </c>
       <c r="U14" s="9" t="s">
-        <v>13</v>
+        <v>137</v>
       </c>
       <c r="V14" s="12"/>
       <c r="W14" s="9" t="s">
-        <v>17</v>
+        <v>142</v>
       </c>
       <c r="X14" s="8">
         <v>46048</v>
@@ -5935,43 +6263,43 @@
         <v>46048</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>179</v>
+        <v>260</v>
       </c>
       <c r="D15" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>168</v>
+        <v>261</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>180</v>
+        <v>262</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>181</v>
+        <v>263</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>13</v>
+        <v>264</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>12</v>
+        <v>265</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>13</v>
+        <v>264</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>13</v>
+        <v>264</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>182</v>
+        <v>266</v>
       </c>
       <c r="M15" s="9" t="s">
         <v>53</v>
       </c>
       <c r="N15" s="8" t="s">
-        <v>183</v>
+        <v>267</v>
       </c>
       <c r="O15" s="9" t="s">
-        <v>184</v>
+        <v>268</v>
       </c>
       <c r="P15" s="8">
         <v>46052</v>
@@ -5980,16 +6308,16 @@
         <v>46051</v>
       </c>
       <c r="R15" s="23" t="s">
-        <v>40</v>
+        <v>269</v>
       </c>
       <c r="S15" s="9" t="s">
-        <v>12</v>
+        <v>265</v>
       </c>
       <c r="T15" s="18">
         <v>8</v>
       </c>
       <c r="U15" s="9" t="s">
-        <v>13</v>
+        <v>264</v>
       </c>
       <c r="V15" s="12"/>
       <c r="W15" s="9" t="s">
@@ -6000,7 +6328,7 @@
       </c>
       <c r="Y15" s="11"/>
       <c r="Z15" s="9" t="s">
-        <v>49</v>
+        <v>270</v>
       </c>
     </row>
     <row r="16" spans="1:26" s="1" customFormat="1" ht="30">
@@ -6011,40 +6339,40 @@
         <v>46048</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>111</v>
+        <v>146</v>
       </c>
       <c r="D16" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>99</v>
+        <v>147</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>112</v>
+        <v>148</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>13</v>
+        <v>150</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>12</v>
+        <v>151</v>
       </c>
       <c r="J16" s="9" t="s">
-        <v>12</v>
+        <v>151</v>
       </c>
       <c r="K16" s="9" t="s">
-        <v>12</v>
+        <v>151</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>114</v>
+        <v>152</v>
       </c>
       <c r="M16" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N16" s="8" t="s">
-        <v>14</v>
+        <v>153</v>
       </c>
       <c r="O16" s="9" t="s">
         <v>20</v>
@@ -6059,19 +6387,19 @@
         <v>20260126001</v>
       </c>
       <c r="S16" s="9" t="s">
-        <v>12</v>
+        <v>151</v>
       </c>
       <c r="T16" s="18">
         <v>6</v>
       </c>
       <c r="U16" s="9" t="s">
-        <v>12</v>
+        <v>151</v>
       </c>
       <c r="V16" s="12" t="s">
-        <v>97</v>
+        <v>154</v>
       </c>
       <c r="W16" s="9" t="s">
-        <v>17</v>
+        <v>155</v>
       </c>
       <c r="X16" s="8">
         <v>46049</v>
@@ -6091,40 +6419,40 @@
         <v>46048</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>111</v>
+        <v>146</v>
       </c>
       <c r="D17" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>99</v>
+        <v>147</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>115</v>
+        <v>156</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>116</v>
+        <v>157</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>12</v>
+        <v>151</v>
       </c>
       <c r="I17" s="9" t="s">
-        <v>12</v>
+        <v>151</v>
       </c>
       <c r="J17" s="9" t="s">
-        <v>12</v>
+        <v>151</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>12</v>
+        <v>151</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>117</v>
+        <v>158</v>
       </c>
       <c r="M17" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N17" s="8" t="s">
-        <v>14</v>
+        <v>153</v>
       </c>
       <c r="O17" s="9" t="s">
         <v>20</v>
@@ -6139,19 +6467,19 @@
         <v>20260126001</v>
       </c>
       <c r="S17" s="9" t="s">
-        <v>12</v>
+        <v>151</v>
       </c>
       <c r="T17" s="18">
         <v>6</v>
       </c>
       <c r="U17" s="9" t="s">
-        <v>12</v>
+        <v>151</v>
       </c>
       <c r="V17" s="12" t="s">
-        <v>97</v>
+        <v>154</v>
       </c>
       <c r="W17" s="9" t="s">
-        <v>17</v>
+        <v>155</v>
       </c>
       <c r="X17" s="8">
         <v>46049</v>
@@ -6171,7 +6499,7 @@
         <v>46048</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>118</v>
+        <v>159</v>
       </c>
       <c r="D18" s="9" t="s">
         <v>39</v>
@@ -6183,28 +6511,28 @@
         <v>45</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>119</v>
+        <v>160</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="L18" s="10" t="s">
-        <v>120</v>
+        <v>162</v>
       </c>
       <c r="M18" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N18" s="8" t="s">
-        <v>14</v>
+        <v>163</v>
       </c>
       <c r="O18" s="9" t="s">
         <v>20</v>
@@ -6219,16 +6547,16 @@
         <v>20260115004</v>
       </c>
       <c r="S18" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="T18" s="18">
         <v>31</v>
       </c>
       <c r="U18" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="V18" s="12" t="s">
-        <v>121</v>
+        <v>165</v>
       </c>
       <c r="W18" s="9"/>
       <c r="X18" s="8"/>
@@ -6247,7 +6575,7 @@
         <v>46048</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>118</v>
+        <v>159</v>
       </c>
       <c r="D19" s="9" t="s">
         <v>43</v>
@@ -6262,25 +6590,25 @@
         <v>43</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="I19" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="L19" s="10" t="s">
-        <v>47</v>
+        <v>166</v>
       </c>
       <c r="M19" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N19" s="8" t="s">
-        <v>14</v>
+        <v>163</v>
       </c>
       <c r="O19" s="9" t="s">
         <v>20</v>
@@ -6295,16 +6623,16 @@
         <v>20260115004</v>
       </c>
       <c r="S19" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="T19" s="18">
         <v>19</v>
       </c>
       <c r="U19" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="V19" s="12" t="s">
-        <v>122</v>
+        <v>167</v>
       </c>
       <c r="W19" s="9"/>
       <c r="X19" s="8"/>
@@ -6323,31 +6651,31 @@
         <v>46049</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>118</v>
+        <v>159</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>123</v>
+        <v>168</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>124</v>
+        <v>169</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>125</v>
+        <v>170</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="L20" s="10" t="s">
         <v>54</v>
@@ -6356,7 +6684,7 @@
         <v>20</v>
       </c>
       <c r="N20" s="8" t="s">
-        <v>14</v>
+        <v>163</v>
       </c>
       <c r="O20" s="9" t="s">
         <v>20</v>
@@ -6371,19 +6699,19 @@
         <v>20260115004</v>
       </c>
       <c r="S20" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="T20" s="18">
         <v>1</v>
       </c>
       <c r="U20" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="V20" s="12" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="W20" s="9" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="X20" s="8">
         <v>46049</v>
@@ -6403,31 +6731,31 @@
         <v>46049</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>118</v>
+        <v>159</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>123</v>
+        <v>168</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>127</v>
+        <v>173</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>128</v>
+        <v>174</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="L21" s="10" t="s">
         <v>54</v>
@@ -6436,7 +6764,7 @@
         <v>20</v>
       </c>
       <c r="N21" s="8" t="s">
-        <v>14</v>
+        <v>163</v>
       </c>
       <c r="O21" s="9" t="s">
         <v>20</v>
@@ -6451,19 +6779,19 @@
         <v>20260115004</v>
       </c>
       <c r="S21" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="T21" s="18">
         <v>1</v>
       </c>
       <c r="U21" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="V21" s="12" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="W21" s="9" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="X21" s="8">
         <v>46049</v>
@@ -6483,31 +6811,31 @@
         <v>46049</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>118</v>
+        <v>159</v>
       </c>
       <c r="D22" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>123</v>
+        <v>168</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>129</v>
+        <v>175</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="J22" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="L22" s="10" t="s">
         <v>54</v>
@@ -6516,7 +6844,7 @@
         <v>20</v>
       </c>
       <c r="N22" s="8" t="s">
-        <v>14</v>
+        <v>163</v>
       </c>
       <c r="O22" s="9" t="s">
         <v>20</v>
@@ -6531,19 +6859,19 @@
         <v>20260115004</v>
       </c>
       <c r="S22" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="T22" s="18">
         <v>1</v>
       </c>
       <c r="U22" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="V22" s="12" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="W22" s="9" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="X22" s="8">
         <v>46049</v>
@@ -6563,31 +6891,31 @@
         <v>46049</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>118</v>
+        <v>159</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>123</v>
+        <v>168</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>131</v>
+        <v>177</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>132</v>
+        <v>178</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="L23" s="10" t="s">
         <v>54</v>
@@ -6596,7 +6924,7 @@
         <v>20</v>
       </c>
       <c r="N23" s="8" t="s">
-        <v>14</v>
+        <v>163</v>
       </c>
       <c r="O23" s="9" t="s">
         <v>20</v>
@@ -6611,19 +6939,19 @@
         <v>20260115004</v>
       </c>
       <c r="S23" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="T23" s="18">
         <v>1</v>
       </c>
       <c r="U23" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="V23" s="12" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="W23" s="9" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="X23" s="8">
         <v>46049</v>
@@ -6643,31 +6971,31 @@
         <v>46049</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>118</v>
+        <v>159</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>123</v>
+        <v>168</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>133</v>
+        <v>179</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>134</v>
+        <v>180</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="J24" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="K24" s="9" t="s">
-        <v>13</v>
+        <v>161</v>
       </c>
       <c r="L24" s="10" t="s">
         <v>54</v>
@@ -6676,7 +7004,7 @@
         <v>20</v>
       </c>
       <c r="N24" s="8" t="s">
-        <v>14</v>
+        <v>163</v>
       </c>
       <c r="O24" s="9" t="s">
         <v>20</v>
@@ -6691,19 +7019,19 @@
         <v>20260115004</v>
       </c>
       <c r="S24" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="T24" s="18">
         <v>1</v>
       </c>
       <c r="U24" s="9" t="s">
-        <v>12</v>
+        <v>164</v>
       </c>
       <c r="V24" s="12" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="W24" s="9" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="X24" s="8">
         <v>46049</v>
@@ -6723,34 +7051,34 @@
         <v>46052</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>135</v>
+        <v>181</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>61</v>
+        <v>182</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>136</v>
+        <v>183</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>137</v>
+        <v>184</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>13</v>
+        <v>185</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>12</v>
+        <v>186</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>13</v>
+        <v>185</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>13</v>
+        <v>185</v>
       </c>
       <c r="L25" s="10" t="s">
-        <v>138</v>
+        <v>187</v>
       </c>
       <c r="M25" s="9" t="s">
         <v>20</v>
@@ -6759,7 +7087,7 @@
         <v>15</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>139</v>
+        <v>188</v>
       </c>
       <c r="P25" s="8">
         <v>46052</v>
@@ -6768,20 +7096,20 @@
         <v>46052</v>
       </c>
       <c r="R25" s="23" t="s">
-        <v>40</v>
+        <v>189</v>
       </c>
       <c r="S25" s="9" t="s">
-        <v>12</v>
+        <v>186</v>
       </c>
       <c r="T25" s="18">
         <v>2.5</v>
       </c>
       <c r="U25" s="9" t="s">
-        <v>13</v>
+        <v>185</v>
       </c>
       <c r="V25" s="12"/>
       <c r="W25" s="9" t="s">
-        <v>17</v>
+        <v>190</v>
       </c>
       <c r="X25" s="8">
         <v>46052</v>
@@ -6799,43 +7127,43 @@
         <v>46056</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>140</v>
+        <v>191</v>
       </c>
       <c r="D26" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>41</v>
+        <v>192</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>141</v>
+        <v>193</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>142</v>
+        <v>194</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>13</v>
+        <v>195</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>12</v>
+        <v>196</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>12</v>
+        <v>196</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>12</v>
+        <v>196</v>
       </c>
       <c r="L26" s="10" t="s">
-        <v>143</v>
+        <v>197</v>
       </c>
       <c r="M26" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N26" s="8" t="s">
-        <v>14</v>
+        <v>198</v>
       </c>
       <c r="O26" s="9" t="s">
-        <v>20</v>
+        <v>199</v>
       </c>
       <c r="P26" s="8">
         <v>46059</v>
@@ -6844,22 +7172,22 @@
         <v>46058</v>
       </c>
       <c r="R26" s="23" t="s">
-        <v>144</v>
+        <v>200</v>
       </c>
       <c r="S26" s="9" t="s">
-        <v>12</v>
+        <v>196</v>
       </c>
       <c r="T26" s="18">
         <v>6</v>
       </c>
       <c r="U26" s="9" t="s">
-        <v>12</v>
+        <v>196</v>
       </c>
       <c r="V26" s="12" t="s">
-        <v>145</v>
+        <v>201</v>
       </c>
       <c r="W26" s="9" t="s">
-        <v>17</v>
+        <v>202</v>
       </c>
       <c r="X26" s="8">
         <v>46058</v>
@@ -6879,31 +7207,31 @@
         <v>46059</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>146</v>
+        <v>203</v>
       </c>
       <c r="D27" s="9" t="s">
         <v>43</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>44</v>
+        <v>204</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>44</v>
+        <v>204</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>147</v>
+        <v>205</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>13</v>
+        <v>206</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>13</v>
+        <v>206</v>
       </c>
       <c r="J27" s="9" t="s">
-        <v>13</v>
+        <v>206</v>
       </c>
       <c r="K27" s="9" t="s">
-        <v>13</v>
+        <v>206</v>
       </c>
       <c r="L27" s="10" t="s">
         <v>47</v>
@@ -6912,7 +7240,7 @@
         <v>20</v>
       </c>
       <c r="N27" s="8" t="s">
-        <v>14</v>
+        <v>207</v>
       </c>
       <c r="O27" s="9" t="s">
         <v>20</v>
@@ -6924,10 +7252,10 @@
         <v>46064</v>
       </c>
       <c r="R27" s="23" t="s">
-        <v>144</v>
+        <v>200</v>
       </c>
       <c r="S27" s="9" t="s">
-        <v>12</v>
+        <v>208</v>
       </c>
       <c r="T27" s="18">
         <v>3</v>
@@ -6936,7 +7264,7 @@
         <v>12</v>
       </c>
       <c r="V27" s="12" t="s">
-        <v>148</v>
+        <v>209</v>
       </c>
       <c r="W27" s="9"/>
       <c r="X27" s="8"/>
@@ -6955,40 +7283,40 @@
         <v>46059</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>146</v>
+        <v>203</v>
       </c>
       <c r="D28" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>123</v>
+        <v>210</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>149</v>
+        <v>211</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>150</v>
+        <v>212</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>12</v>
+        <v>208</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>12</v>
+        <v>208</v>
       </c>
       <c r="J28" s="9" t="s">
-        <v>13</v>
+        <v>206</v>
       </c>
       <c r="K28" s="9" t="s">
-        <v>13</v>
+        <v>206</v>
       </c>
       <c r="L28" s="10" t="s">
-        <v>54</v>
+        <v>213</v>
       </c>
       <c r="M28" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N28" s="8" t="s">
-        <v>14</v>
+        <v>207</v>
       </c>
       <c r="O28" s="9" t="s">
         <v>20</v>
@@ -7000,10 +7328,10 @@
         <v>46064</v>
       </c>
       <c r="R28" s="23" t="s">
-        <v>144</v>
+        <v>200</v>
       </c>
       <c r="S28" s="9" t="s">
-        <v>12</v>
+        <v>208</v>
       </c>
       <c r="T28" s="18">
         <v>3</v>
@@ -7012,10 +7340,10 @@
         <v>12</v>
       </c>
       <c r="V28" s="12" t="s">
-        <v>151</v>
+        <v>214</v>
       </c>
       <c r="W28" s="9" t="s">
-        <v>17</v>
+        <v>215</v>
       </c>
       <c r="X28" s="8">
         <v>46064</v>
@@ -7035,40 +7363,40 @@
         <v>46059</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>146</v>
+        <v>203</v>
       </c>
       <c r="D29" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>123</v>
+        <v>210</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>127</v>
+        <v>216</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>128</v>
+        <v>217</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>13</v>
+        <v>206</v>
       </c>
       <c r="I29" s="9" t="s">
-        <v>12</v>
+        <v>208</v>
       </c>
       <c r="J29" s="9" t="s">
-        <v>13</v>
+        <v>206</v>
       </c>
       <c r="K29" s="9" t="s">
-        <v>13</v>
+        <v>206</v>
       </c>
       <c r="L29" s="10" t="s">
-        <v>54</v>
+        <v>213</v>
       </c>
       <c r="M29" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N29" s="8" t="s">
-        <v>14</v>
+        <v>207</v>
       </c>
       <c r="O29" s="9" t="s">
         <v>20</v>
@@ -7080,10 +7408,10 @@
         <v>46064</v>
       </c>
       <c r="R29" s="23" t="s">
-        <v>144</v>
+        <v>200</v>
       </c>
       <c r="S29" s="9" t="s">
-        <v>12</v>
+        <v>208</v>
       </c>
       <c r="T29" s="18">
         <v>1</v>
@@ -7092,10 +7420,10 @@
         <v>12</v>
       </c>
       <c r="V29" s="12" t="s">
-        <v>151</v>
+        <v>214</v>
       </c>
       <c r="W29" s="9" t="s">
-        <v>17</v>
+        <v>215</v>
       </c>
       <c r="X29" s="8">
         <v>46064</v>
@@ -7115,40 +7443,40 @@
         <v>46059</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>146</v>
+        <v>203</v>
       </c>
       <c r="D30" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>152</v>
+        <v>218</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>153</v>
+        <v>219</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>154</v>
+        <v>220</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>13</v>
+        <v>206</v>
       </c>
       <c r="I30" s="9" t="s">
-        <v>12</v>
+        <v>208</v>
       </c>
       <c r="J30" s="9" t="s">
-        <v>13</v>
+        <v>206</v>
       </c>
       <c r="K30" s="9" t="s">
-        <v>13</v>
+        <v>206</v>
       </c>
       <c r="L30" s="10" t="s">
-        <v>54</v>
+        <v>213</v>
       </c>
       <c r="M30" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N30" s="8" t="s">
-        <v>14</v>
+        <v>207</v>
       </c>
       <c r="O30" s="9" t="s">
         <v>20</v>
@@ -7160,10 +7488,10 @@
         <v>46064</v>
       </c>
       <c r="R30" s="23" t="s">
-        <v>144</v>
+        <v>200</v>
       </c>
       <c r="S30" s="9" t="s">
-        <v>12</v>
+        <v>208</v>
       </c>
       <c r="T30" s="18">
         <v>1</v>
@@ -7172,10 +7500,10 @@
         <v>12</v>
       </c>
       <c r="V30" s="12" t="s">
-        <v>151</v>
+        <v>214</v>
       </c>
       <c r="W30" s="9" t="s">
-        <v>17</v>
+        <v>215</v>
       </c>
       <c r="X30" s="8">
         <v>46064</v>
@@ -7195,40 +7523,40 @@
         <v>46059</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>146</v>
+        <v>203</v>
       </c>
       <c r="D31" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>152</v>
+        <v>218</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>155</v>
+        <v>221</v>
       </c>
       <c r="G31" s="10" t="s">
-        <v>154</v>
+        <v>220</v>
       </c>
       <c r="H31" s="9" t="s">
-        <v>13</v>
+        <v>206</v>
       </c>
       <c r="I31" s="9" t="s">
-        <v>12</v>
+        <v>208</v>
       </c>
       <c r="J31" s="9" t="s">
-        <v>13</v>
+        <v>206</v>
       </c>
       <c r="K31" s="9" t="s">
-        <v>13</v>
+        <v>206</v>
       </c>
       <c r="L31" s="10" t="s">
-        <v>54</v>
+        <v>213</v>
       </c>
       <c r="M31" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N31" s="8" t="s">
-        <v>14</v>
+        <v>207</v>
       </c>
       <c r="O31" s="9" t="s">
         <v>20</v>
@@ -7240,10 +7568,10 @@
         <v>46064</v>
       </c>
       <c r="R31" s="23" t="s">
-        <v>144</v>
+        <v>200</v>
       </c>
       <c r="S31" s="9" t="s">
-        <v>12</v>
+        <v>208</v>
       </c>
       <c r="T31" s="18">
         <v>1</v>
@@ -7252,10 +7580,10 @@
         <v>12</v>
       </c>
       <c r="V31" s="12" t="s">
-        <v>151</v>
+        <v>214</v>
       </c>
       <c r="W31" s="9" t="s">
-        <v>17</v>
+        <v>215</v>
       </c>
       <c r="X31" s="8">
         <v>46064</v>
@@ -7275,43 +7603,43 @@
         <v>46057</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>173</v>
+        <v>252</v>
       </c>
       <c r="D32" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>168</v>
+        <v>244</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>174</v>
+        <v>253</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>175</v>
+        <v>254</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>13</v>
+        <v>247</v>
       </c>
       <c r="I32" s="9" t="s">
-        <v>12</v>
+        <v>248</v>
       </c>
       <c r="J32" s="9" t="s">
-        <v>13</v>
+        <v>247</v>
       </c>
       <c r="K32" s="9" t="s">
-        <v>13</v>
+        <v>247</v>
       </c>
       <c r="L32" s="10" t="s">
-        <v>176</v>
+        <v>255</v>
       </c>
       <c r="M32" s="9" t="s">
         <v>53</v>
       </c>
       <c r="N32" s="8" t="s">
-        <v>14</v>
+        <v>250</v>
       </c>
       <c r="O32" s="9" t="s">
-        <v>38</v>
+        <v>256</v>
       </c>
       <c r="P32" s="8">
         <v>46065</v>
@@ -7320,16 +7648,16 @@
         <v>46064</v>
       </c>
       <c r="R32" s="23" t="s">
-        <v>172</v>
+        <v>251</v>
       </c>
       <c r="S32" s="9" t="s">
-        <v>12</v>
+        <v>248</v>
       </c>
       <c r="T32" s="18">
         <v>20</v>
       </c>
       <c r="U32" s="9" t="s">
-        <v>12</v>
+        <v>248</v>
       </c>
       <c r="V32" s="12" t="s">
         <v>57</v>
@@ -7344,7 +7672,7 @@
         <v>46064</v>
       </c>
       <c r="Z32" s="9" t="s">
-        <v>49</v>
+        <v>257</v>
       </c>
     </row>
     <row r="33" spans="1:26" s="1" customFormat="1" ht="30">
@@ -7355,43 +7683,43 @@
         <v>46057</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>173</v>
+        <v>252</v>
       </c>
       <c r="D33" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>168</v>
+        <v>244</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>177</v>
+        <v>258</v>
       </c>
       <c r="G33" s="10" t="s">
-        <v>178</v>
+        <v>259</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>13</v>
+        <v>247</v>
       </c>
       <c r="I33" s="9" t="s">
-        <v>12</v>
+        <v>248</v>
       </c>
       <c r="J33" s="9" t="s">
-        <v>13</v>
+        <v>247</v>
       </c>
       <c r="K33" s="9" t="s">
-        <v>13</v>
+        <v>247</v>
       </c>
       <c r="L33" s="10" t="s">
-        <v>176</v>
+        <v>255</v>
       </c>
       <c r="M33" s="9" t="s">
         <v>53</v>
       </c>
       <c r="N33" s="8" t="s">
-        <v>14</v>
+        <v>250</v>
       </c>
       <c r="O33" s="9" t="s">
-        <v>38</v>
+        <v>256</v>
       </c>
       <c r="P33" s="8">
         <v>46065</v>
@@ -7400,16 +7728,16 @@
         <v>46064</v>
       </c>
       <c r="R33" s="23" t="s">
-        <v>172</v>
+        <v>251</v>
       </c>
       <c r="S33" s="9" t="s">
-        <v>12</v>
+        <v>248</v>
       </c>
       <c r="T33" s="18">
         <v>20</v>
       </c>
       <c r="U33" s="9" t="s">
-        <v>12</v>
+        <v>248</v>
       </c>
       <c r="V33" s="12" t="s">
         <v>57</v>
@@ -7424,7 +7752,7 @@
         <v>46064</v>
       </c>
       <c r="Z33" s="9" t="s">
-        <v>49</v>
+        <v>257</v>
       </c>
     </row>
     <row r="34" spans="1:26" s="1" customFormat="1" ht="30">
@@ -7435,7 +7763,7 @@
         <v>46065</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>160</v>
+        <v>231</v>
       </c>
       <c r="D34" s="9" t="s">
         <v>36</v>
@@ -7444,31 +7772,31 @@
         <v>41</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>156</v>
+        <v>222</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>157</v>
+        <v>223</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>13</v>
+        <v>224</v>
       </c>
       <c r="I34" s="9" t="s">
-        <v>12</v>
+        <v>225</v>
       </c>
       <c r="J34" s="9" t="s">
-        <v>13</v>
+        <v>224</v>
       </c>
       <c r="K34" s="9" t="s">
-        <v>13</v>
+        <v>224</v>
       </c>
       <c r="L34" s="10" t="s">
-        <v>158</v>
+        <v>226</v>
       </c>
       <c r="M34" s="9" t="s">
         <v>20</v>
       </c>
       <c r="N34" s="8" t="s">
-        <v>14</v>
+        <v>227</v>
       </c>
       <c r="O34" s="9" t="s">
         <v>20</v>
@@ -7480,22 +7808,22 @@
         <v>46065</v>
       </c>
       <c r="R34" s="23" t="s">
-        <v>40</v>
+        <v>228</v>
       </c>
       <c r="S34" s="9" t="s">
-        <v>12</v>
+        <v>225</v>
       </c>
       <c r="T34" s="18">
         <v>4</v>
       </c>
       <c r="U34" s="9" t="s">
-        <v>12</v>
+        <v>225</v>
       </c>
       <c r="V34" s="12" t="s">
-        <v>159</v>
+        <v>229</v>
       </c>
       <c r="W34" s="9" t="s">
-        <v>17</v>
+        <v>230</v>
       </c>
       <c r="X34" s="8">
         <v>46065</v>
@@ -7508,235 +7836,191 @@
       </c>
     </row>
     <row r="35" spans="1:26" s="1" customFormat="1" ht="30">
-      <c r="A35" s="8">
+      <c r="A35" s="16">
         <v>46077</v>
       </c>
-      <c r="B35" s="8">
+      <c r="B35" s="16">
         <v>46078</v>
       </c>
-      <c r="C35" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="D35" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E35" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="F35" s="9" t="s">
-        <v>162</v>
-      </c>
-      <c r="G35" s="10" t="s">
-        <v>163</v>
-      </c>
-      <c r="H35" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="I35" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="J35" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="K35" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="L35" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="M35" s="9" t="s">
+      <c r="C35" s="13" t="s">
+        <v>232</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E35" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="F35" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="G35" s="15" t="s">
+        <v>235</v>
+      </c>
+      <c r="H35" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="I35" s="13" t="s">
+        <v>237</v>
+      </c>
+      <c r="J35" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="K35" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="L35" s="15" t="s">
+        <v>238</v>
+      </c>
+      <c r="M35" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="N35" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="O35" s="9" t="s">
+      <c r="N35" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="O35" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="P35" s="8">
+      <c r="P35" s="16">
         <v>46079</v>
       </c>
-      <c r="Q35" s="8">
+      <c r="Q35" s="16">
         <v>46078</v>
       </c>
-      <c r="R35" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="S35" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="T35" s="18">
+      <c r="R35" s="27" t="s">
+        <v>240</v>
+      </c>
+      <c r="S35" s="13" t="s">
+        <v>237</v>
+      </c>
+      <c r="T35" s="21">
         <v>3</v>
       </c>
-      <c r="U35" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="V35" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="W35" s="9" t="s">
+      <c r="U35" s="13" t="s">
+        <v>237</v>
+      </c>
+      <c r="V35" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="W35" s="13" t="s">
+        <v>242</v>
+      </c>
+      <c r="X35" s="16">
+        <v>46078</v>
+      </c>
+      <c r="Y35" s="14">
+        <v>46078</v>
+      </c>
+      <c r="Z35" s="13" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="36" spans="1:26" s="1" customFormat="1" ht="15">
+      <c r="A36" s="16">
+        <v>45752</v>
+      </c>
+      <c r="B36" s="16">
+        <v>46078</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="D36" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E36" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="F36" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="G36" s="15" t="s">
+        <v>246</v>
+      </c>
+      <c r="H36" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="I36" s="13" t="s">
+        <v>248</v>
+      </c>
+      <c r="J36" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="K36" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="L36" s="15" t="s">
+        <v>249</v>
+      </c>
+      <c r="M36" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="N36" s="16" t="s">
+        <v>250</v>
+      </c>
+      <c r="O36" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="P36" s="16">
+        <v>46079</v>
+      </c>
+      <c r="Q36" s="16">
+        <v>46079</v>
+      </c>
+      <c r="R36" s="27" t="s">
+        <v>251</v>
+      </c>
+      <c r="S36" s="13" t="s">
+        <v>248</v>
+      </c>
+      <c r="T36" s="21">
+        <v>8</v>
+      </c>
+      <c r="U36" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="V36" s="17"/>
+      <c r="W36" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="X35" s="8">
-        <v>46078</v>
-      </c>
-      <c r="Y35" s="11">
-        <v>46078</v>
-      </c>
-      <c r="Z35" s="9" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="36" spans="1:26" s="1" customFormat="1" ht="15">
-      <c r="A36" s="8">
-        <v>45752</v>
-      </c>
-      <c r="B36" s="8">
-        <v>46078</v>
-      </c>
-      <c r="C36" s="9" t="s">
-        <v>167</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E36" s="9" t="s">
-        <v>168</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="G36" s="10" t="s">
-        <v>170</v>
-      </c>
-      <c r="H36" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="I36" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="J36" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="K36" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="L36" s="10" t="s">
-        <v>171</v>
-      </c>
-      <c r="M36" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="N36" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="O36" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="P36" s="8">
+      <c r="X36" s="16">
         <v>46079</v>
       </c>
-      <c r="Q36" s="8">
-        <v>46079</v>
-      </c>
-      <c r="R36" s="23" t="s">
-        <v>172</v>
-      </c>
-      <c r="S36" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="T36" s="18">
-        <v>8</v>
-      </c>
-      <c r="U36" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="V36" s="12"/>
-      <c r="W36" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="X36" s="8">
-        <v>46079</v>
-      </c>
-      <c r="Y36" s="11"/>
-      <c r="Z36" s="9" t="s">
+      <c r="Y36" s="14"/>
+      <c r="Z36" s="13" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="37" spans="1:26" s="1" customFormat="1" ht="30">
-      <c r="A37" s="16">
-        <v>46083</v>
-      </c>
-      <c r="B37" s="16">
-        <v>46083</v>
-      </c>
-      <c r="C37" s="13" t="s">
-        <v>186</v>
-      </c>
+    <row r="37" spans="1:26" s="1" customFormat="1" ht="15">
+      <c r="A37" s="16"/>
+      <c r="B37" s="16"/>
+      <c r="C37" s="13"/>
       <c r="D37" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="E37" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="F37" s="13" t="s">
-        <v>187</v>
-      </c>
-      <c r="G37" s="15" t="s">
-        <v>188</v>
-      </c>
-      <c r="H37" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I37" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="J37" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="K37" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="L37" s="15" t="s">
-        <v>189</v>
-      </c>
-      <c r="M37" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="N37" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="O37" s="13" t="s">
-        <v>190</v>
-      </c>
-      <c r="P37" s="16">
-        <v>46083</v>
-      </c>
-      <c r="Q37" s="16">
-        <v>3.2</v>
-      </c>
-      <c r="R37" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="S37" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="T37" s="21">
-        <v>3</v>
-      </c>
-      <c r="U37" s="13" t="s">
-        <v>13</v>
-      </c>
+      <c r="E37" s="13"/>
+      <c r="F37" s="13"/>
+      <c r="G37" s="15"/>
+      <c r="H37" s="13"/>
+      <c r="I37" s="13"/>
+      <c r="J37" s="13"/>
+      <c r="K37" s="13"/>
+      <c r="L37" s="15"/>
+      <c r="M37" s="13"/>
+      <c r="N37" s="16"/>
+      <c r="O37" s="13"/>
+      <c r="P37" s="16"/>
+      <c r="Q37" s="16"/>
+      <c r="R37" s="27"/>
+      <c r="S37" s="13"/>
+      <c r="T37" s="21"/>
+      <c r="U37" s="13"/>
       <c r="V37" s="17"/>
-      <c r="W37" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="X37" s="16">
-        <v>46083</v>
-      </c>
+      <c r="W37" s="13"/>
+      <c r="X37" s="16"/>
       <c r="Y37" s="14"/>
       <c r="Z37" s="13" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="1:26" s="1" customFormat="1" ht="15">
@@ -7759,7 +8043,7 @@
       <c r="O38" s="13"/>
       <c r="P38" s="16"/>
       <c r="Q38" s="16"/>
-      <c r="R38" s="25"/>
+      <c r="R38" s="27"/>
       <c r="S38" s="13"/>
       <c r="T38" s="21"/>
       <c r="U38" s="13"/>
@@ -7791,7 +8075,7 @@
       <c r="O39" s="13"/>
       <c r="P39" s="16"/>
       <c r="Q39" s="16"/>
-      <c r="R39" s="25"/>
+      <c r="R39" s="27"/>
       <c r="S39" s="13"/>
       <c r="T39" s="21"/>
       <c r="U39" s="13"/>
@@ -7823,7 +8107,7 @@
       <c r="O40" s="13"/>
       <c r="P40" s="16"/>
       <c r="Q40" s="16"/>
-      <c r="R40" s="25"/>
+      <c r="R40" s="27"/>
       <c r="S40" s="13"/>
       <c r="T40" s="21"/>
       <c r="U40" s="13"/>
@@ -7855,7 +8139,7 @@
       <c r="O41" s="13"/>
       <c r="P41" s="16"/>
       <c r="Q41" s="16"/>
-      <c r="R41" s="25"/>
+      <c r="R41" s="27"/>
       <c r="S41" s="13"/>
       <c r="T41" s="21"/>
       <c r="U41" s="13"/>
@@ -7887,7 +8171,7 @@
       <c r="O42" s="13"/>
       <c r="P42" s="16"/>
       <c r="Q42" s="16"/>
-      <c r="R42" s="25"/>
+      <c r="R42" s="27"/>
       <c r="S42" s="13"/>
       <c r="T42" s="21"/>
       <c r="U42" s="13"/>
@@ -7919,7 +8203,7 @@
       <c r="O43" s="13"/>
       <c r="P43" s="16"/>
       <c r="Q43" s="16"/>
-      <c r="R43" s="25"/>
+      <c r="R43" s="27"/>
       <c r="S43" s="13"/>
       <c r="T43" s="21"/>
       <c r="U43" s="13"/>
@@ -7951,7 +8235,7 @@
       <c r="O44" s="13"/>
       <c r="P44" s="16"/>
       <c r="Q44" s="16"/>
-      <c r="R44" s="25"/>
+      <c r="R44" s="27"/>
       <c r="S44" s="13"/>
       <c r="T44" s="21"/>
       <c r="U44" s="13"/>
@@ -7983,7 +8267,7 @@
       <c r="O45" s="13"/>
       <c r="P45" s="16"/>
       <c r="Q45" s="16"/>
-      <c r="R45" s="25"/>
+      <c r="R45" s="27"/>
       <c r="S45" s="13"/>
       <c r="T45" s="21"/>
       <c r="U45" s="13"/>
@@ -8015,7 +8299,7 @@
       <c r="O46" s="13"/>
       <c r="P46" s="16"/>
       <c r="Q46" s="16"/>
-      <c r="R46" s="25"/>
+      <c r="R46" s="27"/>
       <c r="S46" s="13"/>
       <c r="T46" s="21"/>
       <c r="U46" s="13"/>
@@ -8047,7 +8331,7 @@
       <c r="O47" s="13"/>
       <c r="P47" s="16"/>
       <c r="Q47" s="16"/>
-      <c r="R47" s="25"/>
+      <c r="R47" s="27"/>
       <c r="S47" s="13"/>
       <c r="T47" s="21"/>
       <c r="U47" s="13"/>
@@ -8079,7 +8363,7 @@
       <c r="O48" s="13"/>
       <c r="P48" s="16"/>
       <c r="Q48" s="16"/>
-      <c r="R48" s="25"/>
+      <c r="R48" s="27"/>
       <c r="S48" s="13"/>
       <c r="T48" s="21"/>
       <c r="U48" s="13"/>
@@ -8111,7 +8395,7 @@
       <c r="O49" s="13"/>
       <c r="P49" s="16"/>
       <c r="Q49" s="16"/>
-      <c r="R49" s="25"/>
+      <c r="R49" s="27"/>
       <c r="S49" s="13"/>
       <c r="T49" s="21"/>
       <c r="U49" s="13"/>
@@ -8143,7 +8427,7 @@
       <c r="O50" s="13"/>
       <c r="P50" s="16"/>
       <c r="Q50" s="16"/>
-      <c r="R50" s="25"/>
+      <c r="R50" s="27"/>
       <c r="S50" s="13"/>
       <c r="T50" s="21"/>
       <c r="U50" s="13"/>
@@ -8175,7 +8459,7 @@
       <c r="O51" s="13"/>
       <c r="P51" s="16"/>
       <c r="Q51" s="16"/>
-      <c r="R51" s="25"/>
+      <c r="R51" s="27"/>
       <c r="S51" s="13"/>
       <c r="T51" s="21"/>
       <c r="U51" s="13"/>
@@ -8207,7 +8491,7 @@
       <c r="O52" s="13"/>
       <c r="P52" s="16"/>
       <c r="Q52" s="16"/>
-      <c r="R52" s="25"/>
+      <c r="R52" s="27"/>
       <c r="S52" s="13"/>
       <c r="T52" s="21"/>
       <c r="U52" s="13"/>
@@ -8239,7 +8523,7 @@
       <c r="O53" s="13"/>
       <c r="P53" s="16"/>
       <c r="Q53" s="16"/>
-      <c r="R53" s="25"/>
+      <c r="R53" s="27"/>
       <c r="S53" s="13"/>
       <c r="T53" s="21"/>
       <c r="U53" s="13"/>
@@ -8271,7 +8555,7 @@
       <c r="O54" s="13"/>
       <c r="P54" s="16"/>
       <c r="Q54" s="16"/>
-      <c r="R54" s="25"/>
+      <c r="R54" s="27"/>
       <c r="S54" s="13"/>
       <c r="T54" s="21"/>
       <c r="U54" s="13"/>
@@ -8303,7 +8587,7 @@
       <c r="O55" s="13"/>
       <c r="P55" s="16"/>
       <c r="Q55" s="16"/>
-      <c r="R55" s="25"/>
+      <c r="R55" s="27"/>
       <c r="S55" s="13"/>
       <c r="T55" s="21"/>
       <c r="U55" s="13"/>
@@ -8335,7 +8619,7 @@
       <c r="O56" s="13"/>
       <c r="P56" s="16"/>
       <c r="Q56" s="16"/>
-      <c r="R56" s="25"/>
+      <c r="R56" s="27"/>
       <c r="S56" s="13"/>
       <c r="T56" s="21"/>
       <c r="U56" s="13"/>
@@ -8367,7 +8651,7 @@
       <c r="O57" s="13"/>
       <c r="P57" s="16"/>
       <c r="Q57" s="16"/>
-      <c r="R57" s="25"/>
+      <c r="R57" s="27"/>
       <c r="S57" s="13"/>
       <c r="T57" s="21"/>
       <c r="U57" s="13"/>
@@ -8399,7 +8683,7 @@
       <c r="O58" s="13"/>
       <c r="P58" s="16"/>
       <c r="Q58" s="16"/>
-      <c r="R58" s="25"/>
+      <c r="R58" s="27"/>
       <c r="S58" s="13"/>
       <c r="T58" s="21"/>
       <c r="U58" s="13"/>
@@ -8431,7 +8715,7 @@
       <c r="O59" s="13"/>
       <c r="P59" s="16"/>
       <c r="Q59" s="16"/>
-      <c r="R59" s="25"/>
+      <c r="R59" s="27"/>
       <c r="S59" s="13"/>
       <c r="T59" s="21"/>
       <c r="U59" s="13"/>
@@ -8463,7 +8747,7 @@
       <c r="O60" s="13"/>
       <c r="P60" s="16"/>
       <c r="Q60" s="16"/>
-      <c r="R60" s="25"/>
+      <c r="R60" s="27"/>
       <c r="S60" s="13"/>
       <c r="T60" s="21"/>
       <c r="U60" s="13"/>
@@ -8495,7 +8779,7 @@
       <c r="O61" s="13"/>
       <c r="P61" s="16"/>
       <c r="Q61" s="16"/>
-      <c r="R61" s="25"/>
+      <c r="R61" s="27"/>
       <c r="S61" s="13"/>
       <c r="T61" s="21"/>
       <c r="U61" s="13"/>
@@ -8527,7 +8811,7 @@
       <c r="O62" s="13"/>
       <c r="P62" s="16"/>
       <c r="Q62" s="16"/>
-      <c r="R62" s="25"/>
+      <c r="R62" s="27"/>
       <c r="S62" s="13"/>
       <c r="T62" s="21"/>
       <c r="U62" s="13"/>
@@ -8559,7 +8843,7 @@
       <c r="O63" s="13"/>
       <c r="P63" s="16"/>
       <c r="Q63" s="16"/>
-      <c r="R63" s="25"/>
+      <c r="R63" s="27"/>
       <c r="S63" s="13"/>
       <c r="T63" s="21"/>
       <c r="U63" s="13"/>
@@ -8591,7 +8875,7 @@
       <c r="O64" s="13"/>
       <c r="P64" s="16"/>
       <c r="Q64" s="16"/>
-      <c r="R64" s="25"/>
+      <c r="R64" s="27"/>
       <c r="S64" s="13"/>
       <c r="T64" s="21"/>
       <c r="U64" s="13"/>
@@ -8623,7 +8907,7 @@
       <c r="O65" s="13"/>
       <c r="P65" s="16"/>
       <c r="Q65" s="16"/>
-      <c r="R65" s="25"/>
+      <c r="R65" s="27"/>
       <c r="S65" s="13"/>
       <c r="T65" s="21"/>
       <c r="U65" s="13"/>
@@ -8655,7 +8939,7 @@
       <c r="O66" s="13"/>
       <c r="P66" s="16"/>
       <c r="Q66" s="16"/>
-      <c r="R66" s="25"/>
+      <c r="R66" s="27"/>
       <c r="S66" s="13"/>
       <c r="T66" s="21"/>
       <c r="U66" s="13"/>
@@ -8687,7 +8971,7 @@
       <c r="O67" s="13"/>
       <c r="P67" s="16"/>
       <c r="Q67" s="16"/>
-      <c r="R67" s="25"/>
+      <c r="R67" s="27"/>
       <c r="S67" s="13"/>
       <c r="T67" s="21"/>
       <c r="U67" s="13"/>
@@ -8719,7 +9003,7 @@
       <c r="O68" s="13"/>
       <c r="P68" s="16"/>
       <c r="Q68" s="16"/>
-      <c r="R68" s="25"/>
+      <c r="R68" s="27"/>
       <c r="S68" s="13"/>
       <c r="T68" s="21"/>
       <c r="U68" s="13"/>
@@ -8751,7 +9035,7 @@
       <c r="O69" s="13"/>
       <c r="P69" s="16"/>
       <c r="Q69" s="16"/>
-      <c r="R69" s="25"/>
+      <c r="R69" s="27"/>
       <c r="S69" s="13"/>
       <c r="T69" s="21"/>
       <c r="U69" s="13"/>
@@ -8783,7 +9067,7 @@
       <c r="O70" s="13"/>
       <c r="P70" s="16"/>
       <c r="Q70" s="16"/>
-      <c r="R70" s="25"/>
+      <c r="R70" s="27"/>
       <c r="S70" s="13"/>
       <c r="T70" s="21"/>
       <c r="U70" s="13"/>
@@ -8815,7 +9099,7 @@
       <c r="O71" s="13"/>
       <c r="P71" s="16"/>
       <c r="Q71" s="16"/>
-      <c r="R71" s="25"/>
+      <c r="R71" s="27"/>
       <c r="S71" s="13"/>
       <c r="T71" s="21"/>
       <c r="U71" s="13"/>
@@ -8847,7 +9131,7 @@
       <c r="O72" s="13"/>
       <c r="P72" s="16"/>
       <c r="Q72" s="16"/>
-      <c r="R72" s="25"/>
+      <c r="R72" s="27"/>
       <c r="S72" s="13"/>
       <c r="T72" s="21"/>
       <c r="U72" s="13"/>
@@ -8879,7 +9163,7 @@
       <c r="O73" s="13"/>
       <c r="P73" s="16"/>
       <c r="Q73" s="16"/>
-      <c r="R73" s="25"/>
+      <c r="R73" s="27"/>
       <c r="S73" s="13"/>
       <c r="T73" s="21"/>
       <c r="U73" s="13"/>
@@ -8911,7 +9195,7 @@
       <c r="O74" s="13"/>
       <c r="P74" s="16"/>
       <c r="Q74" s="16"/>
-      <c r="R74" s="25"/>
+      <c r="R74" s="27"/>
       <c r="S74" s="13"/>
       <c r="T74" s="21"/>
       <c r="U74" s="13"/>
@@ -8943,7 +9227,7 @@
       <c r="O75" s="13"/>
       <c r="P75" s="16"/>
       <c r="Q75" s="16"/>
-      <c r="R75" s="25"/>
+      <c r="R75" s="27"/>
       <c r="S75" s="13"/>
       <c r="T75" s="21"/>
       <c r="U75" s="13"/>
@@ -8975,7 +9259,7 @@
       <c r="O76" s="13"/>
       <c r="P76" s="16"/>
       <c r="Q76" s="16"/>
-      <c r="R76" s="25"/>
+      <c r="R76" s="27"/>
       <c r="S76" s="13"/>
       <c r="T76" s="21"/>
       <c r="U76" s="13"/>
@@ -9007,7 +9291,7 @@
       <c r="O77" s="13"/>
       <c r="P77" s="16"/>
       <c r="Q77" s="16"/>
-      <c r="R77" s="25"/>
+      <c r="R77" s="27"/>
       <c r="S77" s="13"/>
       <c r="T77" s="21"/>
       <c r="U77" s="13"/>
@@ -9039,7 +9323,7 @@
       <c r="O78" s="13"/>
       <c r="P78" s="16"/>
       <c r="Q78" s="16"/>
-      <c r="R78" s="25"/>
+      <c r="R78" s="27"/>
       <c r="S78" s="13"/>
       <c r="T78" s="21"/>
       <c r="U78" s="13"/>
@@ -9071,7 +9355,7 @@
       <c r="O79" s="13"/>
       <c r="P79" s="16"/>
       <c r="Q79" s="16"/>
-      <c r="R79" s="25"/>
+      <c r="R79" s="27"/>
       <c r="S79" s="13"/>
       <c r="T79" s="21"/>
       <c r="U79" s="13"/>
@@ -9103,7 +9387,7 @@
       <c r="O80" s="13"/>
       <c r="P80" s="16"/>
       <c r="Q80" s="16"/>
-      <c r="R80" s="25"/>
+      <c r="R80" s="27"/>
       <c r="S80" s="13"/>
       <c r="T80" s="21"/>
       <c r="U80" s="13"/>
@@ -9135,7 +9419,7 @@
       <c r="O81" s="13"/>
       <c r="P81" s="16"/>
       <c r="Q81" s="16"/>
-      <c r="R81" s="25"/>
+      <c r="R81" s="27"/>
       <c r="S81" s="13"/>
       <c r="T81" s="21"/>
       <c r="U81" s="13"/>
@@ -9167,7 +9451,7 @@
       <c r="O82" s="13"/>
       <c r="P82" s="16"/>
       <c r="Q82" s="16"/>
-      <c r="R82" s="25"/>
+      <c r="R82" s="27"/>
       <c r="S82" s="13"/>
       <c r="T82" s="21"/>
       <c r="U82" s="13"/>
@@ -9199,7 +9483,7 @@
       <c r="O83" s="13"/>
       <c r="P83" s="16"/>
       <c r="Q83" s="16"/>
-      <c r="R83" s="25"/>
+      <c r="R83" s="27"/>
       <c r="S83" s="13"/>
       <c r="T83" s="21"/>
       <c r="U83" s="13"/>
@@ -9231,7 +9515,7 @@
       <c r="O84" s="13"/>
       <c r="P84" s="16"/>
       <c r="Q84" s="16"/>
-      <c r="R84" s="25"/>
+      <c r="R84" s="27"/>
       <c r="S84" s="13"/>
       <c r="T84" s="21"/>
       <c r="U84" s="13"/>
@@ -9263,7 +9547,7 @@
       <c r="O85" s="13"/>
       <c r="P85" s="16"/>
       <c r="Q85" s="16"/>
-      <c r="R85" s="25"/>
+      <c r="R85" s="27"/>
       <c r="S85" s="13"/>
       <c r="T85" s="21"/>
       <c r="U85" s="13"/>
@@ -9295,7 +9579,7 @@
       <c r="O86" s="13"/>
       <c r="P86" s="16"/>
       <c r="Q86" s="16"/>
-      <c r="R86" s="25"/>
+      <c r="R86" s="27"/>
       <c r="S86" s="13"/>
       <c r="T86" s="21"/>
       <c r="U86" s="13"/>
@@ -9327,7 +9611,7 @@
       <c r="O87" s="13"/>
       <c r="P87" s="16"/>
       <c r="Q87" s="16"/>
-      <c r="R87" s="25"/>
+      <c r="R87" s="27"/>
       <c r="S87" s="13"/>
       <c r="T87" s="21"/>
       <c r="U87" s="13"/>
@@ -9359,7 +9643,7 @@
       <c r="O88" s="13"/>
       <c r="P88" s="16"/>
       <c r="Q88" s="16"/>
-      <c r="R88" s="25"/>
+      <c r="R88" s="27"/>
       <c r="S88" s="13"/>
       <c r="T88" s="21"/>
       <c r="U88" s="13"/>
@@ -9391,7 +9675,7 @@
       <c r="O89" s="13"/>
       <c r="P89" s="16"/>
       <c r="Q89" s="16"/>
-      <c r="R89" s="25"/>
+      <c r="R89" s="27"/>
       <c r="S89" s="13"/>
       <c r="T89" s="21"/>
       <c r="U89" s="13"/>
@@ -9423,7 +9707,7 @@
       <c r="O90" s="13"/>
       <c r="P90" s="16"/>
       <c r="Q90" s="16"/>
-      <c r="R90" s="25"/>
+      <c r="R90" s="27"/>
       <c r="S90" s="13"/>
       <c r="T90" s="21"/>
       <c r="U90" s="13"/>
@@ -9455,7 +9739,7 @@
       <c r="O91" s="13"/>
       <c r="P91" s="16"/>
       <c r="Q91" s="16"/>
-      <c r="R91" s="25"/>
+      <c r="R91" s="27"/>
       <c r="S91" s="13"/>
       <c r="T91" s="21"/>
       <c r="U91" s="13"/>
@@ -9487,7 +9771,7 @@
       <c r="O92" s="13"/>
       <c r="P92" s="16"/>
       <c r="Q92" s="16"/>
-      <c r="R92" s="25"/>
+      <c r="R92" s="27"/>
       <c r="S92" s="13"/>
       <c r="T92" s="21"/>
       <c r="U92" s="13"/>
@@ -9519,7 +9803,7 @@
       <c r="O93" s="13"/>
       <c r="P93" s="16"/>
       <c r="Q93" s="16"/>
-      <c r="R93" s="25"/>
+      <c r="R93" s="27"/>
       <c r="S93" s="13"/>
       <c r="T93" s="21"/>
       <c r="U93" s="13"/>
@@ -9551,7 +9835,7 @@
       <c r="O94" s="13"/>
       <c r="P94" s="16"/>
       <c r="Q94" s="16"/>
-      <c r="R94" s="25"/>
+      <c r="R94" s="27"/>
       <c r="S94" s="13"/>
       <c r="T94" s="21"/>
       <c r="U94" s="13"/>
@@ -9583,7 +9867,7 @@
       <c r="O95" s="13"/>
       <c r="P95" s="16"/>
       <c r="Q95" s="16"/>
-      <c r="R95" s="25"/>
+      <c r="R95" s="27"/>
       <c r="S95" s="13"/>
       <c r="T95" s="21"/>
       <c r="U95" s="13"/>
@@ -9615,7 +9899,7 @@
       <c r="O96" s="13"/>
       <c r="P96" s="16"/>
       <c r="Q96" s="16"/>
-      <c r="R96" s="25"/>
+      <c r="R96" s="27"/>
       <c r="S96" s="13"/>
       <c r="T96" s="21"/>
       <c r="U96" s="13"/>
@@ -9647,7 +9931,7 @@
       <c r="O97" s="13"/>
       <c r="P97" s="16"/>
       <c r="Q97" s="16"/>
-      <c r="R97" s="25"/>
+      <c r="R97" s="27"/>
       <c r="S97" s="13"/>
       <c r="T97" s="21"/>
       <c r="U97" s="13"/>
@@ -9679,7 +9963,7 @@
       <c r="O98" s="13"/>
       <c r="P98" s="16"/>
       <c r="Q98" s="16"/>
-      <c r="R98" s="25"/>
+      <c r="R98" s="27"/>
       <c r="S98" s="13"/>
       <c r="T98" s="21"/>
       <c r="U98" s="13"/>
@@ -9711,7 +9995,7 @@
       <c r="O99" s="13"/>
       <c r="P99" s="16"/>
       <c r="Q99" s="16"/>
-      <c r="R99" s="25"/>
+      <c r="R99" s="27"/>
       <c r="S99" s="13"/>
       <c r="T99" s="21"/>
       <c r="U99" s="13"/>
@@ -9743,7 +10027,7 @@
       <c r="O100" s="13"/>
       <c r="P100" s="16"/>
       <c r="Q100" s="16"/>
-      <c r="R100" s="25"/>
+      <c r="R100" s="27"/>
       <c r="S100" s="13"/>
       <c r="T100" s="21"/>
       <c r="U100" s="13"/>
@@ -9775,7 +10059,7 @@
       <c r="O101" s="13"/>
       <c r="P101" s="16"/>
       <c r="Q101" s="16"/>
-      <c r="R101" s="25"/>
+      <c r="R101" s="27"/>
       <c r="S101" s="13"/>
       <c r="T101" s="21"/>
       <c r="U101" s="13"/>
@@ -9807,7 +10091,7 @@
       <c r="O102" s="13"/>
       <c r="P102" s="16"/>
       <c r="Q102" s="16"/>
-      <c r="R102" s="25"/>
+      <c r="R102" s="27"/>
       <c r="S102" s="13"/>
       <c r="T102" s="21"/>
       <c r="U102" s="13"/>
@@ -9839,7 +10123,7 @@
       <c r="O103" s="13"/>
       <c r="P103" s="16"/>
       <c r="Q103" s="16"/>
-      <c r="R103" s="25"/>
+      <c r="R103" s="27"/>
       <c r="S103" s="13"/>
       <c r="T103" s="21"/>
       <c r="U103" s="13"/>
@@ -9871,7 +10155,7 @@
       <c r="O104" s="13"/>
       <c r="P104" s="16"/>
       <c r="Q104" s="16"/>
-      <c r="R104" s="25"/>
+      <c r="R104" s="27"/>
       <c r="S104" s="13"/>
       <c r="T104" s="21"/>
       <c r="U104" s="13"/>
@@ -9903,7 +10187,7 @@
       <c r="O105" s="13"/>
       <c r="P105" s="16"/>
       <c r="Q105" s="16"/>
-      <c r="R105" s="25"/>
+      <c r="R105" s="27"/>
       <c r="S105" s="13"/>
       <c r="T105" s="21"/>
       <c r="U105" s="13"/>
@@ -9935,7 +10219,7 @@
       <c r="O106" s="13"/>
       <c r="P106" s="16"/>
       <c r="Q106" s="16"/>
-      <c r="R106" s="25"/>
+      <c r="R106" s="27"/>
       <c r="S106" s="13"/>
       <c r="T106" s="21"/>
       <c r="U106" s="13"/>
@@ -9967,7 +10251,7 @@
       <c r="O107" s="13"/>
       <c r="P107" s="16"/>
       <c r="Q107" s="16"/>
-      <c r="R107" s="25"/>
+      <c r="R107" s="27"/>
       <c r="S107" s="13"/>
       <c r="T107" s="21"/>
       <c r="U107" s="13"/>
@@ -9999,7 +10283,7 @@
       <c r="O108" s="13"/>
       <c r="P108" s="16"/>
       <c r="Q108" s="16"/>
-      <c r="R108" s="25"/>
+      <c r="R108" s="27"/>
       <c r="S108" s="13"/>
       <c r="T108" s="21"/>
       <c r="U108" s="13"/>
@@ -10031,7 +10315,7 @@
       <c r="O109" s="13"/>
       <c r="P109" s="16"/>
       <c r="Q109" s="16"/>
-      <c r="R109" s="25"/>
+      <c r="R109" s="27"/>
       <c r="S109" s="13"/>
       <c r="T109" s="21"/>
       <c r="U109" s="13"/>
@@ -10063,7 +10347,7 @@
       <c r="O110" s="13"/>
       <c r="P110" s="16"/>
       <c r="Q110" s="16"/>
-      <c r="R110" s="25"/>
+      <c r="R110" s="27"/>
       <c r="S110" s="13"/>
       <c r="T110" s="21"/>
       <c r="U110" s="13"/>
@@ -10095,7 +10379,7 @@
       <c r="O111" s="13"/>
       <c r="P111" s="16"/>
       <c r="Q111" s="16"/>
-      <c r="R111" s="25"/>
+      <c r="R111" s="27"/>
       <c r="S111" s="13"/>
       <c r="T111" s="21"/>
       <c r="U111" s="13"/>
@@ -10127,7 +10411,7 @@
       <c r="O112" s="13"/>
       <c r="P112" s="16"/>
       <c r="Q112" s="16"/>
-      <c r="R112" s="25"/>
+      <c r="R112" s="27"/>
       <c r="S112" s="13"/>
       <c r="T112" s="21"/>
       <c r="U112" s="13"/>
@@ -10159,7 +10443,7 @@
       <c r="O113" s="13"/>
       <c r="P113" s="16"/>
       <c r="Q113" s="16"/>
-      <c r="R113" s="25"/>
+      <c r="R113" s="27"/>
       <c r="S113" s="13"/>
       <c r="T113" s="21"/>
       <c r="U113" s="13"/>
@@ -10191,7 +10475,7 @@
       <c r="O114" s="13"/>
       <c r="P114" s="16"/>
       <c r="Q114" s="16"/>
-      <c r="R114" s="25"/>
+      <c r="R114" s="27"/>
       <c r="S114" s="13"/>
       <c r="T114" s="21"/>
       <c r="U114" s="13"/>
@@ -10223,7 +10507,7 @@
       <c r="O115" s="13"/>
       <c r="P115" s="16"/>
       <c r="Q115" s="16"/>
-      <c r="R115" s="25"/>
+      <c r="R115" s="27"/>
       <c r="S115" s="13"/>
       <c r="T115" s="21"/>
       <c r="U115" s="13"/>
@@ -10255,7 +10539,7 @@
       <c r="O116" s="13"/>
       <c r="P116" s="16"/>
       <c r="Q116" s="16"/>
-      <c r="R116" s="25"/>
+      <c r="R116" s="27"/>
       <c r="S116" s="13"/>
       <c r="T116" s="21"/>
       <c r="U116" s="13"/>
@@ -10287,7 +10571,7 @@
       <c r="O117" s="13"/>
       <c r="P117" s="16"/>
       <c r="Q117" s="16"/>
-      <c r="R117" s="25"/>
+      <c r="R117" s="27"/>
       <c r="S117" s="13"/>
       <c r="T117" s="21"/>
       <c r="U117" s="13"/>
@@ -10319,7 +10603,7 @@
       <c r="O118" s="13"/>
       <c r="P118" s="16"/>
       <c r="Q118" s="16"/>
-      <c r="R118" s="25"/>
+      <c r="R118" s="27"/>
       <c r="S118" s="13"/>
       <c r="T118" s="21"/>
       <c r="U118" s="13"/>
@@ -10351,7 +10635,7 @@
       <c r="O119" s="13"/>
       <c r="P119" s="16"/>
       <c r="Q119" s="16"/>
-      <c r="R119" s="25"/>
+      <c r="R119" s="27"/>
       <c r="S119" s="13"/>
       <c r="T119" s="21"/>
       <c r="U119" s="13"/>
@@ -10383,7 +10667,7 @@
       <c r="O120" s="13"/>
       <c r="P120" s="16"/>
       <c r="Q120" s="16"/>
-      <c r="R120" s="25"/>
+      <c r="R120" s="27"/>
       <c r="S120" s="13"/>
       <c r="T120" s="21"/>
       <c r="U120" s="13"/>
@@ -10415,7 +10699,7 @@
       <c r="O121" s="13"/>
       <c r="P121" s="16"/>
       <c r="Q121" s="16"/>
-      <c r="R121" s="25"/>
+      <c r="R121" s="27"/>
       <c r="S121" s="13"/>
       <c r="T121" s="21"/>
       <c r="U121" s="13"/>
@@ -10447,7 +10731,7 @@
       <c r="O122" s="13"/>
       <c r="P122" s="16"/>
       <c r="Q122" s="16"/>
-      <c r="R122" s="25"/>
+      <c r="R122" s="27"/>
       <c r="S122" s="13"/>
       <c r="T122" s="21"/>
       <c r="U122" s="13"/>
@@ -10479,7 +10763,7 @@
       <c r="O123" s="13"/>
       <c r="P123" s="16"/>
       <c r="Q123" s="16"/>
-      <c r="R123" s="25"/>
+      <c r="R123" s="27"/>
       <c r="S123" s="13"/>
       <c r="T123" s="21"/>
       <c r="U123" s="13"/>
@@ -10511,7 +10795,7 @@
       <c r="O124" s="13"/>
       <c r="P124" s="16"/>
       <c r="Q124" s="16"/>
-      <c r="R124" s="25"/>
+      <c r="R124" s="27"/>
       <c r="S124" s="13"/>
       <c r="T124" s="21"/>
       <c r="U124" s="13"/>
@@ -10543,7 +10827,7 @@
       <c r="O125" s="13"/>
       <c r="P125" s="16"/>
       <c r="Q125" s="16"/>
-      <c r="R125" s="25"/>
+      <c r="R125" s="27"/>
       <c r="S125" s="13"/>
       <c r="T125" s="21"/>
       <c r="U125" s="13"/>
@@ -10575,7 +10859,7 @@
       <c r="O126" s="13"/>
       <c r="P126" s="16"/>
       <c r="Q126" s="16"/>
-      <c r="R126" s="25"/>
+      <c r="R126" s="27"/>
       <c r="S126" s="13"/>
       <c r="T126" s="21"/>
       <c r="U126" s="13"/>
@@ -10607,7 +10891,7 @@
       <c r="O127" s="13"/>
       <c r="P127" s="16"/>
       <c r="Q127" s="16"/>
-      <c r="R127" s="25"/>
+      <c r="R127" s="27"/>
       <c r="S127" s="13"/>
       <c r="T127" s="21"/>
       <c r="U127" s="13"/>
@@ -10639,7 +10923,7 @@
       <c r="O128" s="13"/>
       <c r="P128" s="16"/>
       <c r="Q128" s="16"/>
-      <c r="R128" s="25"/>
+      <c r="R128" s="27"/>
       <c r="S128" s="13"/>
       <c r="T128" s="21"/>
       <c r="U128" s="13"/>
@@ -10671,7 +10955,7 @@
       <c r="O129" s="13"/>
       <c r="P129" s="16"/>
       <c r="Q129" s="16"/>
-      <c r="R129" s="25"/>
+      <c r="R129" s="27"/>
       <c r="S129" s="13"/>
       <c r="T129" s="21"/>
       <c r="U129" s="13"/>
@@ -10703,7 +10987,7 @@
       <c r="O130" s="13"/>
       <c r="P130" s="16"/>
       <c r="Q130" s="16"/>
-      <c r="R130" s="25"/>
+      <c r="R130" s="27"/>
       <c r="S130" s="13"/>
       <c r="T130" s="21"/>
       <c r="U130" s="13"/>
@@ -10723,11 +11007,11 @@
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Z3:Z130" xr:uid="{07EA4E23-01B0-4721-B111-6565CA64327A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D130" xr:uid="{00000000-0002-0000-0100-000000000000}">
+      <formula1>"程式作廢,程式新增,程式修改,手冊,SA,SD,PM"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Z3:Z130" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"TW,DG"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D130" xr:uid="{4B684569-6E95-4B7D-BE2F-A0085C1FA3A6}">
-      <formula1>"程式作廢,程式新增,程式修改,手冊,SA,SD,PM"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>